<commit_message>
sua luong he thog app ceo1983
</commit_message>
<xml_diff>
--- a/document/TEST_CASES_APP_HIEP_HOI_CHI_TIET.xlsx
+++ b/document/TEST_CASES_APP_HIEP_HOI_CHI_TIET.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="549">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="669">
   <si>
     <t>BÁO CÁO TỔNG QUAN BỘ TEST CASE CHI TIẾT ỨNG DỤNG HIỆP HỘI CEO 1983</t>
   </si>
@@ -32,10 +32,10 @@
     <t>TIẾN ĐỘ MÃ NGUỒN</t>
   </si>
   <si>
-    <t>61 Ca kiểm thử</t>
-  </si>
-  <si>
-    <t>61 Ca [ ] (100%)</t>
+    <t>76 Ca kiểm thử</t>
+  </si>
+  <si>
+    <t>76 Ca [ ] (100%)</t>
   </si>
   <si>
     <t>[ ] (Chờ đánh dấu)</t>
@@ -95,6 +95,9 @@
     <t>Thẻ Hội Viên Thông Minh</t>
   </si>
   <si>
+    <t>4 [ ]</t>
+  </si>
+  <si>
     <t>MOD-04</t>
   </si>
   <si>
@@ -110,36 +113,36 @@
     <t>Quét Mã QR &amp; Kết Nối Realtime</t>
   </si>
   <si>
+    <t>MOD-06</t>
+  </si>
+  <si>
+    <t>Trang Cá Nhân &amp; Đồng Bộ</t>
+  </si>
+  <si>
+    <t>8 [ ]</t>
+  </si>
+  <si>
+    <t>MOD-07</t>
+  </si>
+  <si>
+    <t>Cơ Hội Giao Thương B2B</t>
+  </si>
+  <si>
+    <t>MOD-08</t>
+  </si>
+  <si>
+    <t>Gian Hàng Sản Phẩm</t>
+  </si>
+  <si>
+    <t>MOD-09</t>
+  </si>
+  <si>
+    <t>Sự Kiện &amp; Check-in QR</t>
+  </si>
+  <si>
     <t>5 [ ]</t>
   </si>
   <si>
-    <t>MOD-06</t>
-  </si>
-  <si>
-    <t>Trang Cá Nhân &amp; Đồng Bộ</t>
-  </si>
-  <si>
-    <t>MOD-07</t>
-  </si>
-  <si>
-    <t>Cơ Hội Giao Thương B2B</t>
-  </si>
-  <si>
-    <t>MOD-08</t>
-  </si>
-  <si>
-    <t>Gian Hàng Sản Phẩm</t>
-  </si>
-  <si>
-    <t>MOD-09</t>
-  </si>
-  <si>
-    <t>Sự Kiện &amp; Check-in QR</t>
-  </si>
-  <si>
-    <t>4 [ ]</t>
-  </si>
-  <si>
     <t>MOD-10</t>
   </si>
   <si>
@@ -158,7 +161,7 @@
     <t>Gắn Kết &amp; Tin Nhắn</t>
   </si>
   <si>
-    <t>9 [ ]</t>
+    <t>10 [ ]</t>
   </si>
   <si>
     <t>MOD-13</t>
@@ -1824,6 +1827,411 @@
   </si>
   <si>
     <t>Tính năng Issue 14: Tùy biến vị trí ghế sân khấu trực quan linh hoạt trên sơ đồ khán phòng.</t>
+  </si>
+  <si>
+    <t>TC-PROD-004</t>
+  </si>
+  <si>
+    <t>Menu 3 chấm (...) Chỉnh sửa/Xóa &amp; Upload ảnh thật bài đăng chính chủ</t>
+  </si>
+  <si>
+    <t>Gian Hàng Sản Phẩm (/association/products)</t>
+  </si>
+  <si>
+    <t>Hội viên đã đăng ít nhất 1 sản phẩm của chính mình</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /association/products
+2. Chọn tab "Sản phẩm tôi đăng" hoặc tìm sản phẩm của chính mình
+3. Quan sát góc trên bên phải ảnh/thẻ sản phẩm
+4. Bấm vào icon menu 3 chấm (...)
+5. Chọn "Chỉnh sửa" -&gt; Modal mở ra, chọn ảnh từ máy qua input file, kiểm tra preview ảnh qua resolveMediaUrl
+6. Chọn "Xóa" -&gt; Hộp thoại xác nhận hiển thị và xóa sản phẩm thành công</t>
+  </si>
+  <si>
+    <t>Action click menu (...), File upload image/*, Confirm delete</t>
+  </si>
+  <si>
+    <t>Menu 3 chấm hiển thị chuẩn ở góc trên phải, chỉ hiển thị cho bài đăng chính chủ; upload file ảnh thật hoạt động mượt mà và preview đúng URL; xóa sản phẩm cập nhật danh sách tức thì</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Menu 3 chấm chuẩn UX, lọc song ngữ matchCategory, upload ảnh từ thiết bị.</t>
+  </si>
+  <si>
+    <t>TC-OPP-003</t>
+  </si>
+  <si>
+    <t>Menu 3 chấm (...) Chỉnh sửa/Xóa bài đăng cơ hội chính chủ</t>
+  </si>
+  <si>
+    <t>Cơ Hội Giao Thương (/association/opportunities)</t>
+  </si>
+  <si>
+    <t>Hội viên đã đăng cơ hội giao thương của chính mình</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /association/opportunities
+2. Tìm đến thẻ cơ hội do chính mình đăng
+3. Quan sát góc trên bên phải thẻ
+4. Bấm nút 3 chấm (...) -&gt; Chọn "Chỉnh sửa" hoặc "Xóa"
+5. Kiểm tra chân thẻ không còn các nút inline thô</t>
+  </si>
+  <si>
+    <t>Action click menu (...), Edit / Delete opportunity</t>
+  </si>
+  <si>
+    <t>Menu 3 chấm hiển thị ở góc trên phải, hỗ trợ sửa và xóa cơ hội, chân thẻ gọn gàng không bị vỡ dòng</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Tinh gọn thẻ cơ hội, đưa hành động vào dropdown 3 chấm.</t>
+  </si>
+  <si>
+    <t>TC-EVT-005</t>
+  </si>
+  <si>
+    <t>Trang chủ hiển thị tối đa 5 sự kiện tỷ lệ ngang &amp; Danh sách sự kiện tinh gọn overlay</t>
+  </si>
+  <si>
+    <t>Trang chủ (/association) &amp; Danh sách sự kiện (/association/events)</t>
+  </si>
+  <si>
+    <t>Hệ thống có các sự kiện đang diễn ra hoặc sắp tới</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở Trang chủ /association -&gt; Kiểm tra khối Sự kiện sắp tới hiển thị tối đa 5 sự kiện
+2. Quan sát tỷ lệ ảnh poster ngang aspect-[4/3] sm:aspect-[16/10]
+3. Kiểm tra nút "Xem tất cả" kèm icon ChevronRight (thay cho ••• cũ)
+4. Bấm vào để chuyển sang /association/events
+5. Kiểm tra danh sách sự kiện: Toàn bộ Tiêu đề, Countdown timer và nút "Xem chi tiết" nằm gọn gàng bên trong overlay chân poster, không có text rác bên ngoài</t>
+  </si>
+  <si>
+    <t>Navigation /association -&gt; /association/events</t>
+  </si>
+  <si>
+    <t>Trang chủ hiển thị 5 sự kiện ngang chuẩn điện ảnh, nút Xem tất cả trang nhã; trang sự kiện tinh gọn 100% thông tin trong poster overlay</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Chuẩn hóa thẩm mỹ sự kiện C-Level, tỷ lệ ngang điện ảnh.</t>
+  </si>
+  <si>
+    <t>TC-AVT-001</t>
+  </si>
+  <si>
+    <t>Đồng bộ ảnh đại diện thời gian thực giữa Profile và Home qua Event Bus</t>
+  </si>
+  <si>
+    <t>Trang Cá Nhân (/association/profile) &amp; Trang Chủ (/association)</t>
+  </si>
+  <si>
+    <t>Hội viên đã đăng nhập và đang ở tab Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở tab Cá nhân /association/profile
+2. Bấm đổi avatar và tải ảnh đại diện mới
+3. Chuyển ngay sang tab Trang chủ /association mà không reload trang
+4. Quan sát Avatar dập viền nổi trên thẻ VIP trang chủ và trên Header</t>
+  </si>
+  <si>
+    <t>Upload avatar mới</t>
+  </si>
+  <si>
+    <t>Ảnh đại diện trên Trang chủ và Header lập tức cập nhật ảnh mới đồng bộ 100% nhờ event bus vba_member_avatar_updated mà không cần F5</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Cơ chế reactive event bus vba_member_avatar_updated tức thời.</t>
+  </si>
+  <si>
+    <t>TC-PRF-007</t>
+  </si>
+  <si>
+    <t>Gỡ bỏ icon dấu cộng (+) thừa trên dòng "Quản lý Danh thiếp số"</t>
+  </si>
+  <si>
+    <t>Trang Cá Nhân (/association/profile)</t>
+  </si>
+  <si>
+    <t>Đang ở tab Profile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /association/profile
+2. Cuộn đến dòng mục "Quản lý Danh thiếp số"
+3. Quan sát góc bên phải của dòng mục</t>
+  </si>
+  <si>
+    <t>Visual inspect item "Quản lý Danh thiếp số"</t>
+  </si>
+  <si>
+    <t>Dòng mục chỉ hiển thị mũi tên chevron điều hướng sang trang danh thiếp, ĐÃ GỠ BỎ HOÀN TOÀN nút dấu cộng (+) gây hiểu nhầm tạo thêm thẻ</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Chuẩn hóa UX menu cá nhân theo yêu cầu khách hàng.</t>
+  </si>
+  <si>
+    <t>TC-PRF-008</t>
+  </si>
+  <si>
+    <t>Căn giữa tuyệt đối Modal chi tiết hội viên MemberProfileModal trên Mobile</t>
+  </si>
+  <si>
+    <t>Modal MemberProfileModal (/association/members)</t>
+  </si>
+  <si>
+    <t>Mở ứng dụng trên điện thoại di động hoặc Responsive Mode (375px - 414px)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở danh bạ hội viên /association/members
+2. Bấm vào một hội viên bất kỳ để mở Modal chi tiết
+3. Quan sát vị trí hiển thị của hộp thoại modal trên màn hình điện thoại</t>
+  </si>
+  <si>
+    <t>Mobile viewport, Open member profile modal</t>
+  </si>
+  <si>
+    <t>Modal căn chính xác 100% ở giữa màn hình theo cả trục dọc và ngang, không bị lệch sát mép trên hoặc tràn viền đáy</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Cấu trúc lưới fail-safe grid place-items-center w-full h-[100dvh] min-h-[100dvh] my-auto.</t>
+  </si>
+  <si>
+    <t>TC-SCAN-003</t>
+  </si>
+  <si>
+    <t>Quét QR trực tiếp bằng HTML5 in-app scanner, loại bỏ Google Play Code Scanner native</t>
+  </si>
+  <si>
+    <t>Modal Quét QR (/association/card &amp; AssociationQrScanModal)</t>
+  </si>
+  <si>
+    <t>Thiết bị có camera (Android/iOS hoặc Web browser)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Bấm mở modal Quét QR (hoặc tab Quét QR trong Thẻ hội viên)
+2. Cho phép quyền truy cập camera
+3. Quan sát khung ngắm camera WebRTC in-app hiển thị ngay lập tức
+4. Đưa mã QR vào khung ngắm để quét</t>
+  </si>
+  <si>
+    <t>Camera stream, QR code scan</t>
+  </si>
+  <si>
+    <t>Camera in-app bật tức thì mượt mà, nhận diện mã QR thành công, hoàn toàn không gọi AndroidNative.scanQr, không bị đơ/văng trên thiết bị thiếu Google Play Services</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Gỡ bỏ hoàn toàn phụ thuộc Google Play Code Scanner, dùng 100% camera HTML5.</t>
+  </si>
+  <si>
+    <t>TC-MSG-010</t>
+  </si>
+  <si>
+    <t>Xóa cuộc trò chuyện bền vững qua blacklist client-side &amp; Xóa tin nhắn phía tôi trong localMessages</t>
+  </si>
+  <si>
+    <t>Màn hình Tin nhắn (/association/messages)</t>
+  </si>
+  <si>
+    <t>Có các cuộc trò chuyện và tin nhắn trong hộp thư</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /association/messages
+2. Vuốt sang trái hoặc nhấn giữ vào một cuộc trò chuyện -&gt; Chọn "Xóa cuộc trò chuyện"
+3. Xác nhận xóa -&gt; Cuộc trò chuyện biến mất
+4. F5 hoặc tải lại trang -&gt; Kiểm tra cuộc trò chuyện KHÔNG bị xuất hiện trở lại
+5. Mở một thread chat, nhấn giữ tin nhắn -&gt; Chọn "Xóa ở phía tôi"
+6. Tin nhắn biến mất ngay lập tức và không còn trong localMessages</t>
+  </si>
+  <si>
+    <t>Action delete conversation &amp; delete message for me</t>
+  </si>
+  <si>
+    <t>Cuộc trò chuyện bị xóa được lưu vào blacklist vba_deleted_convs và bị lọc vĩnh viễn; xóa tin nhắn phía tôi cập nhật triệt để cả UI và localStorage</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Khắc phục lỗi hồi sinh cuộc trò chuyện sau khi tải lại trang.</t>
+  </si>
+  <si>
+    <t>TC-CARD-004</t>
+  </si>
+  <si>
+    <t>Chuẩn hóa màu sắc Modal chụp danh thiếp Trắng &amp; Xanh Navy #003B95 viền vàng &amp; Toast thông báo</t>
+  </si>
+  <si>
+    <t>Modal Chụp Danh Thiếp (AssociationCardCaptureModal) &amp; Toast UI (sonner.tsx)</t>
+  </si>
+  <si>
+    <t>Tại màn hình quản lý danh thiếp số /association/business-cards</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Bấm nút "Chụp quét danh thiếp"
+2. Quan sát màu sắc nền và viền của Modal
+3. Thực hiện một hành động thành công bất kỳ (Lưu thẻ, copy mã, v.v.) để kích hoạt Toast thông báo</t>
+  </si>
+  <si>
+    <t>Open Card Capture Modal, Trigger Toast</t>
+  </si>
+  <si>
+    <t>Modal chuyển sang phong cách Trắng &amp; Xanh Navy (#003B95) viền vàng kim Amber Gold sang trọng (loại bỏ màu tối #0C1322); Toast hiển thị chuẩn màu Navy &amp; Gold</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Chuẩn hóa nhận diện màu sắc C-Level CEO 1983.</t>
+  </si>
+  <si>
+    <t>TC-CRM-003</t>
+  </si>
+  <si>
+    <t>Phân quyền Sidebar CRM ẩn các nhóm menu không có quyền (network, businessConnect, system)</t>
+  </si>
+  <si>
+    <t>Sidebar Web CRM (/dashboard, /members, v.v.)</t>
+  </si>
+  <si>
+    <t>Đăng nhập với các tài khoản vai trò Trưởng ban hoặc nhân viên</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Đăng nhập tài khoản không có quyền Platform Admin / IT System
+2. Quan sát dải menu Sidebar bên trái
+3. Kiểm tra các nhóm menu: Mạng lưới (network), Business Connect và Hệ thống (system)</t>
+  </si>
+  <si>
+    <t>Role-based access check on Sidebar</t>
+  </si>
+  <si>
+    <t>Các nhóm menu và mục con vượt quyền bị ẩn hoàn toàn, chỉ hiển thị đúng các phân hệ được phân quyền</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Tăng cường bảo mật phân quyền đa cấp trên Web CRM.</t>
+  </si>
+  <si>
+    <t>TC-CRM-004</t>
+  </si>
+  <si>
+    <t>Tạo cơ hội giao thương CRM hỗ trợ upload ảnh từ máy &amp; Đồng bộ trường ảnh</t>
+  </si>
+  <si>
+    <t>Quản lý Cơ hội CRM (/opportunities)</t>
+  </si>
+  <si>
+    <t>Đang ở trang Quản lý Cơ hội CRM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /opportunities -&gt; Bấm nút "Tạo cơ hội mới"
+2. Trong modal tạo cơ hội, quan sát mục Tải ảnh
+3. Chọn một file ảnh từ máy tính -&gt; Xem trước ảnh hiển thị rõ nét
+4. Điền đầy đủ thông tin và bấm Lưu cơ hội</t>
+  </si>
+  <si>
+    <t>File upload image, New opportunity form data</t>
+  </si>
+  <si>
+    <t>Hệ thống hỗ trợ upload file ảnh thật, hiển thị preview ngay trong modal, lưu trữ và đồng bộ trường image/imageUrl lên hệ thống</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Đồng bộ tính năng tải ảnh cơ hội giữa Web CRM và Mobile App.</t>
+  </si>
+  <si>
+    <t>TC-CRM-005</t>
+  </si>
+  <si>
+    <t>Gửi nhắc phí hội viên CRM (kết nối handleRemind trên Card và Row)</t>
+  </si>
+  <si>
+    <t>Quản lý Hội Phí CRM (/fees)</t>
+  </si>
+  <si>
+    <t>Có các hóa đơn hội phí chưa thanh toán (unpaid/pending)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /fees
+2. Chuyển sang dạng thẻ (Card view) hoặc dạng bảng (Table row view)
+3. Tìm hóa đơn chưa thanh toán -&gt; Bấm nút "Nhắc phí"
+4. Quan sát phản hồi của hệ thống</t>
+  </si>
+  <si>
+    <t>Click "Nhắc phí" button on Card / Row</t>
+  </si>
+  <si>
+    <t>Hệ thống kích hoạt hàm handleRemind, hiển thị toast thông báo gửi lời nhắc thành công đến hội viên kèm tên và mã hội viên chính xác</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Gắn kết nối sự kiện nhắc phí đồng bộ cả giao diện thẻ và bảng.</t>
+  </si>
+  <si>
+    <t>TC-CRM-006</t>
+  </si>
+  <si>
+    <t>Khắc phục cột tài khoản bị để trống trong danh sách hội phí CRM</t>
+  </si>
+  <si>
+    <t>Có danh sách hóa đơn hội phí từ backend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /fees
+2. Quan sát cột "Hội viên / Tài khoản" trong bảng danh sách
+3. Kiểm tra các dòng hóa đơn</t>
+  </si>
+  <si>
+    <t>Table render on /fees</t>
+  </si>
+  <si>
+    <t>Cột tài khoản hiển thị đầy đủ thông tin (Mã hội viên, Họ tên, SĐT), KHÔNG BỊ TRỐNG RỖNG nhờ logic fallback kép trong admin.service.ts</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Fallback logic an toàn cho invoice member accounts và joins.</t>
+  </si>
+  <si>
+    <t>TC-CRM-007</t>
+  </si>
+  <si>
+    <t>Lưu trữ trạng thái đóng phí Doanh nghiệp CRM vào Database &amp; Toggle nhanh</t>
+  </si>
+  <si>
+    <t>Quản lý Doanh Nghiệp CRM (/companies)</t>
+  </si>
+  <si>
+    <t>Đang ở trang Quản lý Doanh nghiệp CRM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /companies
+2. Quan sát cột "Hội phí" trong bảng và badge trạng thái trên thẻ doanh nghiệp
+3. Sử dụng bộ lọc "Hội phí" (Tất cả, Đã đóng phí, Chưa đóng phí)
+4. Bấm nút gạt / toggle trạng thái đóng phí trên một doanh nghiệp
+5. Tải lại trang để kiểm tra</t>
+  </si>
+  <si>
+    <t>Toggle fee status, Filter by feePaid</t>
+  </si>
+  <si>
+    <t>Trạng thái đóng phí feePaid và feeYear được lưu trực tiếp vào cơ sở dữ liệu PostgreSQL qua SQL UPDATE; toggle hoạt động mượt mà và bảo lưu sau khi F5</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Quản lý hội phí doanh nghiệp đồng bộ 100% database.</t>
+  </si>
+  <si>
+    <t>TC-CRM-008</t>
+  </si>
+  <si>
+    <t>Sơ đồ rạp chiếu CinemaSeatingMap mở rộng canvas h-[640px], clamp kéo ghế &amp; Thêm hàng ghế dưới</t>
+  </si>
+  <si>
+    <t>Sơ đồ Chỗ Ngồi CRM (/events/seating)</t>
+  </si>
+  <si>
+    <t>Mở sơ đồ CinemaSeatingMap dạng Tiệc (Banquet) và Rạp chiếu (Cinema)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /events/seating
+2. Chuyển sang chế độ Sơ đồ Tiệc (Banquet tables) -&gt; Kiểm tra canvas mở rộng chiều cao h-[640px]
+3. Thử kéo bàn tiệc/ghế xuống sát đáy canvas -&gt; Tọa độ được clamp an toàn tại tối đa 95%, không bị rơi mất
+4. Chuyển sang chế độ Sơ đồ Khán phòng (Cinema rows) -&gt; Kiểm tra khoảng đệm đáy pb-16 min-h-[300px]
+5. Bấm nút "+ Thêm hàng ghế bên dưới" -&gt; Hàng ghế mới được thêm vào đáy sơ đồ</t>
+  </si>
+  <si>
+    <t>Drag banquet tables, Click "+ Thêm hàng ghế bên dưới"</t>
+  </si>
+  <si>
+    <t>Canvas rộng rãi h-[640px], kéo thả không bao giờ bị văng khỏi vùng nhìn thấy, thêm hàng ghế bên dưới hoạt động trực quan chính xác</t>
+  </si>
+  <si>
+    <t>Tính năng Issue 128: Tối ưu trải nghiệm kéo thả sơ đồ rạp chiếu và bàn tiệc sự kiện.</t>
   </si>
 </sst>
 </file>
@@ -2562,10 +2970,10 @@
         <v>26</v>
       </c>
       <c r="D12" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F12" s="13" t="s">
         <v>20</v>
@@ -2576,16 +2984,16 @@
     </row>
     <row r="13" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D13" s="13">
         <v>2</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>20</v>
@@ -2596,16 +3004,16 @@
     </row>
     <row r="14" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D14" s="13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="F14" s="13" t="s">
         <v>20</v>
@@ -2622,10 +3030,10 @@
         <v>34</v>
       </c>
       <c r="D15" s="13">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="F15" s="13" t="s">
         <v>20</v>
@@ -2636,16 +3044,16 @@
     </row>
     <row r="16" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D16" s="13">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F16" s="13" t="s">
         <v>20</v>
@@ -2656,16 +3064,16 @@
     </row>
     <row r="17" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B17" s="11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C17" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D17" s="13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E17" s="14" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F17" s="13" t="s">
         <v>20</v>
@@ -2676,16 +3084,16 @@
     </row>
     <row r="18" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B18" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C18" s="12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D18" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F18" s="13" t="s">
         <v>20</v>
@@ -2696,16 +3104,16 @@
     </row>
     <row r="19" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B19" s="11" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C19" s="12" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D19" s="13">
         <v>2</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F19" s="13" t="s">
         <v>20</v>
@@ -2716,16 +3124,16 @@
     </row>
     <row r="20" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B20" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D20" s="13">
         <v>2</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F20" s="13" t="s">
         <v>20</v>
@@ -2736,16 +3144,16 @@
     </row>
     <row r="21" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B21" s="11" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D21" s="13">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F21" s="13" t="s">
         <v>20</v>
@@ -2756,16 +3164,16 @@
     </row>
     <row r="22" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B22" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D22" s="13">
         <v>2</v>
       </c>
       <c r="E22" s="14" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F22" s="13" t="s">
         <v>20</v>
@@ -2776,10 +3184,10 @@
     </row>
     <row r="23" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B23" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D23" s="13">
         <v>3</v>
@@ -2796,16 +3204,16 @@
     </row>
     <row r="24" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B24" s="11" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D24" s="13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F24" s="13" t="s">
         <v>20</v>
@@ -2816,16 +3224,16 @@
     </row>
     <row r="25" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B25" s="11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D25" s="13">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>24</v>
+        <v>42</v>
       </c>
       <c r="F25" s="13" t="s">
         <v>20</v>
@@ -2836,16 +3244,16 @@
     </row>
     <row r="26" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B26" s="11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D26" s="13">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="F26" s="13" t="s">
         <v>20</v>
@@ -2856,7 +3264,7 @@
     </row>
     <row r="29" ht="26" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B29" s="16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
@@ -2866,7 +3274,7 @@
     </row>
     <row r="30" ht="28" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B30" s="17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C30" s="17"/>
       <c r="D30" s="17"/>
@@ -2876,7 +3284,7 @@
     </row>
     <row r="31" ht="28" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B31" s="17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
@@ -2886,7 +3294,7 @@
     </row>
     <row r="32" ht="28" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B32" s="17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C32" s="17"/>
       <c r="D32" s="17"/>
@@ -2910,7 +3318,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:L65"/>
+  <dimension ref="B2:L80"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -2929,7 +3337,7 @@
   <sheetData>
     <row r="2" ht="36" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="18" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -2944,2172 +3352,2697 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="19" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I4" s="20" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="L4" s="20" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="21" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C5" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G5" s="22" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H5" s="22" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I5" s="22" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K5" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L5" s="22" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="21" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F6" s="22" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H6" s="22" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I6" s="22" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K6" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L6" s="22" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="21" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C7" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G7" s="22" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H7" s="22" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="I7" s="22" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K7" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L7" s="22" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="21" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C8" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G8" s="22" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I8" s="22" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K8" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L8" s="22" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="21" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C9" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H9" s="22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I9" s="22" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K9" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L9" s="22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="21" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C10" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F10" s="22" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G10" s="22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H10" s="22" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I10" s="22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K10" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L10" s="22" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="21" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C11" s="22" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G11" s="22" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H11" s="22" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K11" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L11" s="22" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="21" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C12" s="22" t="s">
         <v>23</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F12" s="22" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H12" s="22" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I12" s="22" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K12" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L12" s="22" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="21" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C13" s="22" t="s">
         <v>23</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F13" s="22" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G13" s="22" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H13" s="22" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I13" s="22" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K13" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L13" s="22" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="21" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C14" s="22" t="s">
         <v>26</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F14" s="22" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G14" s="22" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H14" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I14" s="22" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K14" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L14" s="22" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="21" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C15" s="22" t="s">
         <v>26</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F15" s="22" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G15" s="22" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H15" s="22" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I15" s="22" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K15" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L15" s="22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="21" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C16" s="22" t="s">
         <v>26</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F16" s="22" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="G16" s="22" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H16" s="22" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="I16" s="22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K16" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L16" s="22" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="21" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F17" s="22" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="G17" s="22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H17" s="22" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I17" s="22" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="J17" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K17" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="22" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="21" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F18" s="22" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G18" s="22" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H18" s="22" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="I18" s="22" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J18" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K18" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L18" s="22" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="21" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G19" s="22" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H19" s="22" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I19" s="22" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K19" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L19" s="22" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="21" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G20" s="22" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H20" s="22" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I20" s="22" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K20" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L20" s="22" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="21" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F21" s="22" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G21" s="22" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H21" s="22" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="I21" s="22" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="J21" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K21" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L21" s="22" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="21" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F22" s="22" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G22" s="22" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H22" s="22" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="I22" s="22" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="J22" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K22" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L22" s="22" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="21" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F23" s="22" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H23" s="22" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I23" s="22" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="J23" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K23" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L23" s="22" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="21" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C24" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F24" s="22" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G24" s="22" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H24" s="22" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I24" s="22" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J24" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K24" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L24" s="22" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="21" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C25" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F25" s="22" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G25" s="22" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H25" s="22" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I25" s="22" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J25" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K25" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L25" s="22" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="26" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="21" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C26" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D26" s="22" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F26" s="22" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G26" s="22" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="H26" s="22" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="I26" s="22" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J26" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K26" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L26" s="22" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="27" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="21" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C27" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F27" s="22" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H27" s="22" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="I27" s="22" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="J27" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K27" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L27" s="22" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="28" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="21" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C28" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D28" s="22" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F28" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H28" s="22" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="I28" s="22" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="J28" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K28" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L28" s="22" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="29" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="21" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C29" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D29" s="22" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F29" s="22" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="H29" s="22" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="I29" s="22" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="J29" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K29" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L29" s="22" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="30" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="21" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D30" s="22" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F30" s="22" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G30" s="22" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="H30" s="22" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="I30" s="22" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J30" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K30" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L30" s="22" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="21" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D31" s="22" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F31" s="22" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G31" s="22" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="H31" s="22" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="I31" s="22" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J31" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K31" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L31" s="22" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="32" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="21" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D32" s="22" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F32" s="22" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G32" s="22" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="H32" s="22" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="I32" s="22" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="J32" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K32" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L32" s="22" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="33" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="21" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D33" s="22" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F33" s="22" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="G33" s="22" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="H33" s="22" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="I33" s="22" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="J33" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K33" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L33" s="22" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
     </row>
     <row r="34" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="21" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F34" s="22" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="G34" s="22" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H34" s="22" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="I34" s="22" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J34" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K34" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L34" s="22" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="35" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="21" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D35" s="22" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F35" s="22" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="G35" s="22" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="H35" s="22" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="I35" s="22" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="J35" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K35" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L35" s="22" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
     </row>
     <row r="36" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="21" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D36" s="22" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F36" s="22" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G36" s="22" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="H36" s="22" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="I36" s="22" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="J36" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K36" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L36" s="22" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="37" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="21" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D37" s="22" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F37" s="22" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G37" s="22" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="H37" s="22" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="I37" s="22" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="J37" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K37" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L37" s="22" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="38" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="21" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D38" s="22" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E38" s="22" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F38" s="22" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G38" s="22" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="H38" s="22" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="I38" s="22" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="J38" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K38" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L38" s="22" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="39" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="21" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D39" s="22" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F39" s="22" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G39" s="22" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="H39" s="22" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="I39" s="22" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="J39" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K39" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L39" s="22" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="40" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="21" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D40" s="22" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="E40" s="22" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F40" s="22" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G40" s="22" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H40" s="22" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="I40" s="22" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J40" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K40" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L40" s="22" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="41" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="21" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D41" s="22" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="F41" s="22" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="G41" s="22" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="H41" s="22" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="I41" s="22" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="J41" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K41" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L41" s="22" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
     </row>
     <row r="42" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="21" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E42" s="22" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F42" s="22" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G42" s="22" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="H42" s="22" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="I42" s="22" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J42" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K42" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L42" s="22" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
     </row>
     <row r="43" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="21" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D43" s="22" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F43" s="22" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G43" s="22" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="H43" s="22" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="I43" s="22" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="J43" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K43" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L43" s="22" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
     </row>
     <row r="44" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="21" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D44" s="22" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E44" s="22" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F44" s="22" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="H44" s="22" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="I44" s="22" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J44" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K44" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L44" s="22" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
     </row>
     <row r="45" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="21" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D45" s="22" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F45" s="22" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="G45" s="22" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="H45" s="22" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="I45" s="22" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="J45" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K45" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L45" s="22" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
     <row r="46" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="21" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D46" s="22" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E46" s="22" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F46" s="22" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="G46" s="22" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="H46" s="22" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="I46" s="22" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="J46" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K46" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L46" s="22" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="47" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="21" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D47" s="22" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E47" s="22" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F47" s="22" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G47" s="22" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="H47" s="22" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="I47" s="22" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="J47" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K47" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L47" s="22" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="48" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="21" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D48" s="22" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E48" s="22" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F48" s="22" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="G48" s="22" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="H48" s="22" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="I48" s="22" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="J48" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K48" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L48" s="22" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
     </row>
     <row r="49" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B49" s="21" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D49" s="22" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="E49" s="22" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F49" s="22" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G49" s="22" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="H49" s="22" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="I49" s="22" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="J49" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K49" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L49" s="22" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="50" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B50" s="21" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D50" s="22" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F50" s="22" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G50" s="22" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="H50" s="22" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="I50" s="22" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="J50" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K50" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L50" s="22" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="51" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B51" s="21" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D51" s="22" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E51" s="22" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F51" s="22" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G51" s="22" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="H51" s="22" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="I51" s="22" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="J51" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K51" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L51" s="22" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="52" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B52" s="21" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D52" s="22" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E52" s="22" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F52" s="22" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G52" s="22" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="H52" s="22" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="I52" s="22" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="J52" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K52" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L52" s="22" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
     </row>
     <row r="53" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B53" s="21" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="C53" s="22" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D53" s="22" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E53" s="22" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F53" s="22" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="G53" s="22" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="H53" s="22" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="I53" s="22" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="J53" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K53" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L53" s="22" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
     </row>
     <row r="54" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B54" s="21" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D54" s="22" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E54" s="22" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F54" s="22" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G54" s="22" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="H54" s="22" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="I54" s="22" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="J54" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K54" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L54" s="22" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
     </row>
     <row r="55" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B55" s="21" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="C55" s="22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D55" s="22" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E55" s="22" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F55" s="22" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="G55" s="22" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="H55" s="22" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="I55" s="22" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J55" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K55" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L55" s="22" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
     </row>
     <row r="56" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B56" s="21" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D56" s="22" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E56" s="22" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F56" s="22" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="G56" s="22" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="H56" s="22" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="I56" s="22" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="J56" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K56" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L56" s="22" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="57" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B57" s="21" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="C57" s="22" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D57" s="22" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E57" s="22" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F57" s="22" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="G57" s="22" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="H57" s="22" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="I57" s="22" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J57" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K57" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L57" s="22" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="58" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B58" s="21" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C58" s="22" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D58" s="22" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E58" s="22" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F58" s="22" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G58" s="22" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="H58" s="22" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="I58" s="22" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J58" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K58" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L58" s="22" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="59" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B59" s="21" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="C59" s="22" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D59" s="22" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="E59" s="22" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="F59" s="22" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="G59" s="22" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="H59" s="22" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="I59" s="22" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="J59" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K59" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L59" s="22" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
     </row>
     <row r="60" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B60" s="21" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="C60" s="22" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D60" s="22" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="E60" s="22" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F60" s="22" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G60" s="22" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="H60" s="22" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="I60" s="22" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="J60" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K60" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L60" s="22" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
     </row>
     <row r="61" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B61" s="21" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="C61" s="22" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D61" s="22" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E61" s="22" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F61" s="22" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="G61" s="22" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="H61" s="22" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="I61" s="22" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="J61" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K61" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L61" s="22" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
     </row>
     <row r="62" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B62" s="21" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="C62" s="22" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D62" s="22" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E62" s="22" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F62" s="22" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="G62" s="22" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="H62" s="22" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="I62" s="22" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="J62" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K62" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L62" s="22" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
     </row>
     <row r="63" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B63" s="21" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="C63" s="22" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D63" s="22" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E63" s="22" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="F63" s="22" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="G63" s="22" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="H63" s="22" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="I63" s="22" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="J63" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K63" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L63" s="22" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
     </row>
     <row r="64" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B64" s="21" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D64" s="22" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E64" s="22" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="F64" s="22" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="G64" s="22" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="H64" s="22" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="I64" s="22" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="J64" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K64" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L64" s="22" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="65" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B65" s="21" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D65" s="22" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E65" s="22" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F65" s="22" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="G65" s="22" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="H65" s="22" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="I65" s="22" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="J65" s="23" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K65" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L65" s="22" t="s">
-        <v>548</v>
+        <v>549</v>
+      </c>
+    </row>
+    <row r="66" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B66" s="21" t="s">
+        <v>550</v>
+      </c>
+      <c r="C66" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="D66" s="22" t="s">
+        <v>551</v>
+      </c>
+      <c r="E66" s="22" t="s">
+        <v>552</v>
+      </c>
+      <c r="F66" s="22" t="s">
+        <v>553</v>
+      </c>
+      <c r="G66" s="22" t="s">
+        <v>554</v>
+      </c>
+      <c r="H66" s="22" t="s">
+        <v>555</v>
+      </c>
+      <c r="I66" s="22" t="s">
+        <v>556</v>
+      </c>
+      <c r="J66" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K66" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L66" s="22" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="67" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B67" s="21" t="s">
+        <v>558</v>
+      </c>
+      <c r="C67" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="D67" s="22" t="s">
+        <v>559</v>
+      </c>
+      <c r="E67" s="22" t="s">
+        <v>560</v>
+      </c>
+      <c r="F67" s="22" t="s">
+        <v>561</v>
+      </c>
+      <c r="G67" s="22" t="s">
+        <v>562</v>
+      </c>
+      <c r="H67" s="22" t="s">
+        <v>563</v>
+      </c>
+      <c r="I67" s="22" t="s">
+        <v>564</v>
+      </c>
+      <c r="J67" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K67" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L67" s="22" t="s">
+        <v>565</v>
+      </c>
+    </row>
+    <row r="68" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B68" s="21" t="s">
+        <v>566</v>
+      </c>
+      <c r="C68" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="D68" s="22" t="s">
+        <v>567</v>
+      </c>
+      <c r="E68" s="22" t="s">
+        <v>568</v>
+      </c>
+      <c r="F68" s="22" t="s">
+        <v>569</v>
+      </c>
+      <c r="G68" s="22" t="s">
+        <v>570</v>
+      </c>
+      <c r="H68" s="22" t="s">
+        <v>571</v>
+      </c>
+      <c r="I68" s="22" t="s">
+        <v>572</v>
+      </c>
+      <c r="J68" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K68" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L68" s="22" t="s">
+        <v>573</v>
+      </c>
+    </row>
+    <row r="69" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B69" s="21" t="s">
+        <v>574</v>
+      </c>
+      <c r="C69" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D69" s="22" t="s">
+        <v>575</v>
+      </c>
+      <c r="E69" s="22" t="s">
+        <v>576</v>
+      </c>
+      <c r="F69" s="22" t="s">
+        <v>577</v>
+      </c>
+      <c r="G69" s="22" t="s">
+        <v>578</v>
+      </c>
+      <c r="H69" s="22" t="s">
+        <v>579</v>
+      </c>
+      <c r="I69" s="22" t="s">
+        <v>580</v>
+      </c>
+      <c r="J69" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K69" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L69" s="22" t="s">
+        <v>581</v>
+      </c>
+    </row>
+    <row r="70" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B70" s="21" t="s">
+        <v>582</v>
+      </c>
+      <c r="C70" s="22" t="s">
+        <v>34</v>
+      </c>
+      <c r="D70" s="22" t="s">
+        <v>583</v>
+      </c>
+      <c r="E70" s="22" t="s">
+        <v>584</v>
+      </c>
+      <c r="F70" s="22" t="s">
+        <v>585</v>
+      </c>
+      <c r="G70" s="22" t="s">
+        <v>586</v>
+      </c>
+      <c r="H70" s="22" t="s">
+        <v>587</v>
+      </c>
+      <c r="I70" s="22" t="s">
+        <v>588</v>
+      </c>
+      <c r="J70" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K70" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L70" s="22" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="71" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B71" s="21" t="s">
+        <v>590</v>
+      </c>
+      <c r="C71" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="D71" s="22" t="s">
+        <v>591</v>
+      </c>
+      <c r="E71" s="22" t="s">
+        <v>592</v>
+      </c>
+      <c r="F71" s="22" t="s">
+        <v>593</v>
+      </c>
+      <c r="G71" s="22" t="s">
+        <v>594</v>
+      </c>
+      <c r="H71" s="22" t="s">
+        <v>595</v>
+      </c>
+      <c r="I71" s="22" t="s">
+        <v>596</v>
+      </c>
+      <c r="J71" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K71" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L71" s="22" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="72" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B72" s="21" t="s">
+        <v>598</v>
+      </c>
+      <c r="C72" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="D72" s="22" t="s">
+        <v>599</v>
+      </c>
+      <c r="E72" s="22" t="s">
+        <v>600</v>
+      </c>
+      <c r="F72" s="22" t="s">
+        <v>601</v>
+      </c>
+      <c r="G72" s="22" t="s">
+        <v>602</v>
+      </c>
+      <c r="H72" s="22" t="s">
+        <v>603</v>
+      </c>
+      <c r="I72" s="22" t="s">
+        <v>604</v>
+      </c>
+      <c r="J72" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K72" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L72" s="22" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="73" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B73" s="21" t="s">
+        <v>606</v>
+      </c>
+      <c r="C73" s="22" t="s">
+        <v>48</v>
+      </c>
+      <c r="D73" s="22" t="s">
+        <v>607</v>
+      </c>
+      <c r="E73" s="22" t="s">
+        <v>608</v>
+      </c>
+      <c r="F73" s="22" t="s">
+        <v>609</v>
+      </c>
+      <c r="G73" s="22" t="s">
+        <v>610</v>
+      </c>
+      <c r="H73" s="22" t="s">
+        <v>611</v>
+      </c>
+      <c r="I73" s="22" t="s">
+        <v>612</v>
+      </c>
+      <c r="J73" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K73" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L73" s="22" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="74" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B74" s="21" t="s">
+        <v>614</v>
+      </c>
+      <c r="C74" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D74" s="22" t="s">
+        <v>615</v>
+      </c>
+      <c r="E74" s="22" t="s">
+        <v>616</v>
+      </c>
+      <c r="F74" s="22" t="s">
+        <v>617</v>
+      </c>
+      <c r="G74" s="22" t="s">
+        <v>618</v>
+      </c>
+      <c r="H74" s="22" t="s">
+        <v>619</v>
+      </c>
+      <c r="I74" s="22" t="s">
+        <v>620</v>
+      </c>
+      <c r="J74" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K74" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L74" s="22" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="75" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B75" s="21" t="s">
+        <v>622</v>
+      </c>
+      <c r="C75" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="D75" s="22" t="s">
+        <v>623</v>
+      </c>
+      <c r="E75" s="22" t="s">
+        <v>624</v>
+      </c>
+      <c r="F75" s="22" t="s">
+        <v>625</v>
+      </c>
+      <c r="G75" s="22" t="s">
+        <v>626</v>
+      </c>
+      <c r="H75" s="22" t="s">
+        <v>627</v>
+      </c>
+      <c r="I75" s="22" t="s">
+        <v>628</v>
+      </c>
+      <c r="J75" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K75" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L75" s="22" t="s">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="76" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B76" s="21" t="s">
+        <v>630</v>
+      </c>
+      <c r="C76" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="D76" s="22" t="s">
+        <v>631</v>
+      </c>
+      <c r="E76" s="22" t="s">
+        <v>632</v>
+      </c>
+      <c r="F76" s="22" t="s">
+        <v>633</v>
+      </c>
+      <c r="G76" s="22" t="s">
+        <v>634</v>
+      </c>
+      <c r="H76" s="22" t="s">
+        <v>635</v>
+      </c>
+      <c r="I76" s="22" t="s">
+        <v>636</v>
+      </c>
+      <c r="J76" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K76" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L76" s="22" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="77" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B77" s="21" t="s">
+        <v>638</v>
+      </c>
+      <c r="C77" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="D77" s="22" t="s">
+        <v>639</v>
+      </c>
+      <c r="E77" s="22" t="s">
+        <v>640</v>
+      </c>
+      <c r="F77" s="22" t="s">
+        <v>641</v>
+      </c>
+      <c r="G77" s="22" t="s">
+        <v>642</v>
+      </c>
+      <c r="H77" s="22" t="s">
+        <v>643</v>
+      </c>
+      <c r="I77" s="22" t="s">
+        <v>644</v>
+      </c>
+      <c r="J77" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K77" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L77" s="22" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="78" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B78" s="21" t="s">
+        <v>646</v>
+      </c>
+      <c r="C78" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="D78" s="22" t="s">
+        <v>647</v>
+      </c>
+      <c r="E78" s="22" t="s">
+        <v>640</v>
+      </c>
+      <c r="F78" s="22" t="s">
+        <v>648</v>
+      </c>
+      <c r="G78" s="22" t="s">
+        <v>649</v>
+      </c>
+      <c r="H78" s="22" t="s">
+        <v>650</v>
+      </c>
+      <c r="I78" s="22" t="s">
+        <v>651</v>
+      </c>
+      <c r="J78" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K78" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L78" s="22" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="79" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B79" s="21" t="s">
+        <v>653</v>
+      </c>
+      <c r="C79" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="D79" s="22" t="s">
+        <v>654</v>
+      </c>
+      <c r="E79" s="22" t="s">
+        <v>655</v>
+      </c>
+      <c r="F79" s="22" t="s">
+        <v>656</v>
+      </c>
+      <c r="G79" s="22" t="s">
+        <v>657</v>
+      </c>
+      <c r="H79" s="22" t="s">
+        <v>658</v>
+      </c>
+      <c r="I79" s="22" t="s">
+        <v>659</v>
+      </c>
+      <c r="J79" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K79" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L79" s="22" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="80" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B80" s="21" t="s">
+        <v>661</v>
+      </c>
+      <c r="C80" s="22" t="s">
+        <v>59</v>
+      </c>
+      <c r="D80" s="22" t="s">
+        <v>662</v>
+      </c>
+      <c r="E80" s="22" t="s">
+        <v>663</v>
+      </c>
+      <c r="F80" s="22" t="s">
+        <v>664</v>
+      </c>
+      <c r="G80" s="22" t="s">
+        <v>665</v>
+      </c>
+      <c r="H80" s="22" t="s">
+        <v>666</v>
+      </c>
+      <c r="I80" s="22" t="s">
+        <v>667</v>
+      </c>
+      <c r="J80" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="K80" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L80" s="22" t="s">
+        <v>668</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new config ceo ,crm,vione
</commit_message>
<xml_diff>
--- a/document/TEST_CASES_APP_HIEP_HOI_CHI_TIET.xlsx
+++ b/document/TEST_CASES_APP_HIEP_HOI_CHI_TIET.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="669">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1066" uniqueCount="739">
   <si>
     <t>BÁO CÁO TỔNG QUAN BỘ TEST CASE CHI TIẾT ỨNG DỤNG HIỆP HỘI CEO 1983</t>
   </si>
@@ -32,10 +32,10 @@
     <t>TIẾN ĐỘ MÃ NGUỒN</t>
   </si>
   <si>
-    <t>76 Ca kiểm thử</t>
-  </si>
-  <si>
-    <t>76 Ca [ ] (100%)</t>
+    <t>83 Ca kiểm thử</t>
+  </si>
+  <si>
+    <t>83 Ca [ ] (100%)</t>
   </si>
   <si>
     <t>[ ] (Chờ đánh dấu)</t>
@@ -192,6 +192,51 @@
   </si>
   <si>
     <t>Quản Trị CRM &amp; Sơ Đồ Khán Phòng</t>
+  </si>
+  <si>
+    <t>MOD-18</t>
+  </si>
+  <si>
+    <t>Hạ Tầng &amp; DevOps HTTPS</t>
+  </si>
+  <si>
+    <t>1 [ ]</t>
+  </si>
+  <si>
+    <t>MOD-19</t>
+  </si>
+  <si>
+    <t>Quản Trị Sự Kiện CRM</t>
+  </si>
+  <si>
+    <t>MOD-20</t>
+  </si>
+  <si>
+    <t>Biểu Quyết &amp; Bầu Cử Đại Hội</t>
+  </si>
+  <si>
+    <t>MOD-21</t>
+  </si>
+  <si>
+    <t>Sự Kiện &amp; Quay Số May Mắn</t>
+  </si>
+  <si>
+    <t>MOD-22</t>
+  </si>
+  <si>
+    <t>Sàn Thương Mại &amp; Gian Hàng</t>
+  </si>
+  <si>
+    <t>MOD-23</t>
+  </si>
+  <si>
+    <t>Sàn Cơ Hội Giao Thương B2B</t>
+  </si>
+  <si>
+    <t>MOD-24</t>
+  </si>
+  <si>
+    <t>Ứng Dụng PWA &amp; Mobile iOS</t>
   </si>
   <si>
     <t>📋 NGUYÊN TẮC KIỂM THỬ: TOÀN BỘ Ô KIỂM [ ] ĐỂ TRỐNG ĐỂ NGHIỆM THU THỰC TẾ</t>
@@ -1713,7 +1758,7 @@
     <t>Fee notification payload</t>
   </si>
   <si>
-    <t>Bong bóng tin nhắn hiển thị số tiền niên liễm và nút "Thanh toán ngay qua VietQR"</t>
+    <t>Bong bóng tin nhắn hiển thị số tiền hội phí và nút "Thanh toán ngay qua VietQR"</t>
   </si>
   <si>
     <t>Hóa đơn nhắc nợ trực quan.</t>
@@ -2232,6 +2277,205 @@
   </si>
   <si>
     <t>Tính năng Issue 128: Tối ưu trải nghiệm kéo thả sơ đồ rạp chiếu và bàn tiệc sự kiện.</t>
+  </si>
+  <si>
+    <t>TC-REQ-001</t>
+  </si>
+  <si>
+    <t>Cấu hình SSL Nginx Reverse Proxy &amp; Fast Deploy HTTPS (Ports 5443/5444)</t>
+  </si>
+  <si>
+    <t>Server Dev (14.225.217.232)</t>
+  </si>
+  <si>
+    <t>Nginx SSL Docker Compose và chứng chỉ SAN đã triển khai</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Chạy deploy/ssl/deploy-ssl.ps1 hoặc fast-deploy.ps1 -EnableHttps
+2. Mở trình duyệt truy cập https://14.225.217.232:5443 (Web CRM)
+3. Mở trình duyệt truy cập https://14.225.217.232:5444/association (App Hiệp hội)
+4. Kiểm tra giao thức bảo mật HTTPS và phản hồi API</t>
+  </si>
+  <si>
+    <t>HTTPS Port 5443 / 5444, SSL SAN Cert</t>
+  </si>
+  <si>
+    <t>Cả Web CRM và App Hiệp hội tải mượt mà qua HTTPS, chứng chỉ SAN bao quát IP và sslip.io, API NestJS kết nối ổn định</t>
+  </si>
+  <si>
+    <t>Hỗ trợ cả HTTP và HTTPS thông qua Nginx Reverse Proxy an toàn.</t>
+  </si>
+  <si>
+    <t>TC-REQ-002</t>
+  </si>
+  <si>
+    <t>Tạo Sự Kiện CRM &amp; Tự Động Điền Bố Cục Text &amp; Banner Riêng Theo Loại Sự Kiện</t>
+  </si>
+  <si>
+    <t>Tạo Sự Kiện CRM (/events/new, EventWizard)</t>
+  </si>
+  <si>
+    <t>Đăng nhập CRM bằng quyền Quản trị viên</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /events/new -&gt; Bước 1 "Thông tin cơ bản"
+2. Bấm chọn loại sự kiện "Diễn đàn" (Forum) -&gt; Quan sát Tiêu đề, Tagline, Banner preview, Sức chứa tự động điền mẫu chuyên nghiệp
+3. Đổi sang loại "Workshop" -&gt; Quan sát nội dung và banner đổi sang mẫu Workshop chuyên sâu
+4. Đổi sang loại "Kết nối" (Networking) -&gt; Quan sát nội dung đổi sang Dạ tiệc Doanh nhân
+5. Đổi sang loại "Đào tạo" (Training) -&gt; Quan sát nội dung đổi sang Masterclass Doanh trí
+6. Quan sát khung "Xem trước Banner &amp; Bố cục Sự kiện"</t>
+  </si>
+  <si>
+    <t>Chọn eventType trong EventWizard</t>
+  </si>
+  <si>
+    <t>Tự động điền text nội dung, tagline, sức chứa, địa điểm và hiển thị banner preview riêng biệt khớp 100% từng loại sự kiện</t>
+  </si>
+  <si>
+    <t>Tối ưu trải nghiệm tạo sự kiện cho Admin CRM với bố cục banner động.</t>
+  </si>
+  <si>
+    <t>TC-REQ-003</t>
+  </si>
+  <si>
+    <t>Tạo Biểu Quyết CRM tự động đẩy thông báo thời gian thực về App Hiệp Hội</t>
+  </si>
+  <si>
+    <t>Biểu Quyết CRM (/voting) &amp; Thông Báo App (/association/notifications)</t>
+  </si>
+  <si>
+    <t>Admin tạo phiên biểu quyết mới trên CRM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Trên Web CRM /voting, bấm "Tạo biểu quyết mới"
+2. Nhập tiêu đề, các phương án lựa chọn và lưu phiên
+3. Mở App Hiệp hội với tài khoản hội viên
+4. Quan sát chuông thông báo và danh sách thông báo
+5. Bấm vào thông báo biểu quyết có nút "Tham gia biểu quyết ngay"</t>
+  </si>
+  <si>
+    <t>Tạo phiên voting trên CRM</t>
+  </si>
+  <si>
+    <t>Thông báo đẩy tức thì về App Hiệp hội, hiển thị thẻ biểu quyết tương tác, bấm vào mở ngay modal bầu chọn trực tiếp</t>
+  </si>
+  <si>
+    <t>Liên kết luồng realtime giữa Web CRM và App Hiệp hội.</t>
+  </si>
+  <si>
+    <t>TC-REQ-004</t>
+  </si>
+  <si>
+    <t>Đăng ký vé sinh Số May Mắn ngẫu nhiên (#XXXX) &amp; Quay thưởng Lucky Draw gửi thông báo chúc mừng</t>
+  </si>
+  <si>
+    <t>Đăng ký sự kiện App (/association/events) &amp; Quay thưởng CRM (/voting)</t>
+  </si>
+  <si>
+    <t>Có sự kiện mở đăng ký vé</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Hội viên mở sự kiện trên App Hiệp hội -&gt; Bấm "Đăng ký vé tham gia"
+2. Quan sát hộp thoại xác nhận: Hiển thị "Số may mắn của bạn: #XXXX"
+3. Mở tab Vé của tôi / Lịch sử check-in: Thẻ vé lưu trữ số may mắn định danh
+4. Trên CRM /voting -&gt; Mở module "Quay số may mắn (Lucky Draw)"
+5. Chọn sự kiện và bấm "Bắt đầu quay số"
+6. Hệ thống quay ngẫu nhiên các số may mắn từ danh sách vé đã đăng ký và chọn người trúng
+7. Admin bấm "Gửi thông báo trúng" -&gt; App của người trúng nhận thông báo Chúc mừng thẻ vàng</t>
+  </si>
+  <si>
+    <t>Event registration, Lucky draw spin, Win notification</t>
+  </si>
+  <si>
+    <t>Mỗi vé tự động sinh số ngẫu nhiên 4 chữ số; CRM quay số chính xác theo danh sách vé thực tế; người trúng nhận thông báo vinh danh tức thời</t>
+  </si>
+  <si>
+    <t>Đã backfill số may mắn cho toàn bộ đăng ký cũ, hỗ trợ trọn vẹn chương trình gala sự kiện.</t>
+  </si>
+  <si>
+    <t>TC-REQ-005</t>
+  </si>
+  <si>
+    <t>Sàn thương mại điện tử Luxury: Header tìm kiếm, menu danh mục, bộ lọc, đăng SP &amp; 3 Section phân trang</t>
+  </si>
+  <si>
+    <t>Đã đăng nhập App Hiệp hội</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /association/products
+2. Quan sát Header: Icon Menu danh mục (LayoutGrid) bên trái, Thanh tìm kiếm ở giữa, Icon Bộ lọc và nút "Đăng SP" bên phải
+3. Bấm Icon Menu danh mục -&gt; Menu trượt sổ xuống chọn nhanh ngành hàng
+4. Cuộn xuống quan sát 3 Section: 1) "Sản phẩm mới đăng", 2) "Sản phẩm được xem nhiều nhất", 3) "Doanh nghiệp nổi bật nhất"
+5. Thử bấm phân trang "Trang trước / Trang sau" ở từng Section
+6. Bấm "Xem gian hàng" ở Section 3 -&gt; Mở Showroom giới thiệu doanh nghiệp và các sản phẩm niêm yết</t>
+  </si>
+  <si>
+    <t>Category menu click, Search keyword, Pagination next/prev, View storefront</t>
+  </si>
+  <si>
+    <t>Bố cục chuẩn sàn thương mại điện tử sang trọng; 3 section phân trang độc lập mượt mà; 1 hội viên đại diện cho 1 công ty có gian hàng riêng biệt</t>
+  </si>
+  <si>
+    <t>Nâng cấp toàn diện thẩm mỹ và trải nghiệm thương mại B2B nội khối.</t>
+  </si>
+  <si>
+    <t>TC-REQ-006</t>
+  </si>
+  <si>
+    <t>Bảng Tin Trao Cơ Hội: Phân Trang, Tăng Lượt Xem Realtime &amp; Xem Danh Sách Người Quan Tâm Kèm Call/Email/Chat</t>
+  </si>
+  <si>
+    <t>Màn hình Trao Cơ Hội (/association/opportunities)</t>
+  </si>
+  <si>
+    <t>Có các bài đăng cơ hội giao thương trên hệ thống</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở /association/opportunities -&gt; Quan sát giao diện dạng bảng tin chuyên nghiệp
+2. Bấm chuyển trang phân trang ở chân danh sách (5 bài / trang)
+3. Người dùng B bấm vào xem chi tiết bài đăng của Người dùng A -&gt; Lượt xem tăng lên 1 (POST /opportunities/:id/view)
+4. Người dùng B bấm "Quan tâm"
+5. Người dùng A (chủ bài đăng) mở bài viết của mình -&gt; Thấy khu vực "Hội viên đã quan tâm (X)"
+6. Người dùng A bấm nút Gọi điện (tel), Gửi email (mailto) hoặc Nhắn tin (chuyển sang /messages)</t>
+  </si>
+  <si>
+    <t>Click view detail, Click interest, Owner views interested members list</t>
+  </si>
+  <si>
+    <t>Bảng tin phân trang chuẩn mực; đếm lượt xem chuẩn xác khi xem chi tiết; chủ bài đăng nắm bắt đầy đủ thông tin đối tác quan tâm và liên hệ tức thời</t>
+  </si>
+  <si>
+    <t>Tối đa hóa hiệu quả kết nối và xúc tiến hợp đồng giữa các hội viên.</t>
+  </si>
+  <si>
+    <t>TC-REQ-007</t>
+  </si>
+  <si>
+    <t>Cài đặt PWA trên iPhone/iPad qua Safari Add to Home Screen &amp; Chạy toàn màn hình Offline</t>
+  </si>
+  <si>
+    <t>Trình duyệt Safari trên iOS &amp; Trình duyệt Chrome trên Android</t>
+  </si>
+  <si>
+    <t>Mở đường dẫn /association trên thiết bị di động iOS Safari</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Mở Safari trên iPhone truy cập /association
+2. Quan sát thanh thông báo hướng dẫn cài đặt iOS (IosInstallPrompt) xuất hiện trang nhã ở đáy màn hình
+3. Làm theo hướng dẫn: Bấm nút Share (Chia sẻ) ở thanh điều hướng Safari
+4. Cuộn xuống chọn "Thêm vào MH chính" (Add to Home Screen)
+5. Nhấn "Thêm"
+6. Quay về màn hình chính iPhone -&gt; Biểu tượng App CEO 1983 xuất hiện sắc nét
+7. Nhấn mở app từ màn hình chính -&gt; Ứng dụng chạy toàn màn hình standalone, không có thanh URL Safari</t>
+  </si>
+  <si>
+    <t>iOS Safari, Add to Home Screen, Standalone PWA launch</t>
+  </si>
+  <si>
+    <t>Cài đặt thành công PWA trên iOS, icon chuẩn retina, mở app toàn màn hình mượt mà như ứng dụng Native, hỗ trợ bộ nhớ đệm qua Service Worker</t>
+  </si>
+  <si>
+    <t>Đáp ứng trọn vẹn nhu cầu gửi link cho người dùng iOS trải nghiệm ứng dụng hiệp hội.</t>
   </si>
 </sst>
 </file>
@@ -2837,7 +3081,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:G32"/>
+  <dimension ref="B2:G39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -3262,54 +3506,194 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" ht="26" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B29" s="16" t="s">
+    <row r="27" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B27" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
-      <c r="G29" s="16"/>
-    </row>
-    <row r="30" ht="28" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B30" s="17" t="s">
+      <c r="C27" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C30" s="17"/>
-      <c r="D30" s="17"/>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17"/>
-    </row>
-    <row r="31" ht="28" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B31" s="17" t="s">
+      <c r="D27" s="13">
+        <v>1</v>
+      </c>
+      <c r="E27" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
-    </row>
-    <row r="32" ht="28" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B32" s="17" t="s">
+      <c r="F27" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G27" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B28" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="C32" s="17"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
+      <c r="C28" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" s="13">
+        <v>1</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B29" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D29" s="13">
+        <v>1</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G29" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B30" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D30" s="13">
+        <v>1</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G30" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="31" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B31" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="D31" s="13">
+        <v>1</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G31" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="32" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B32" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D32" s="13">
+        <v>1</v>
+      </c>
+      <c r="E32" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G32" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="33" ht="24" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B33" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D33" s="13">
+        <v>1</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="G33" s="15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36" ht="26" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B36" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="C36" s="16"/>
+      <c r="D36" s="16"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="16"/>
+      <c r="G36" s="16"/>
+    </row>
+    <row r="37" ht="28" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B37" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="C37" s="17"/>
+      <c r="D37" s="17"/>
+      <c r="E37" s="17"/>
+      <c r="F37" s="17"/>
+      <c r="G37" s="17"/>
+    </row>
+    <row r="38" ht="28" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B38" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="C38" s="17"/>
+      <c r="D38" s="17"/>
+      <c r="E38" s="17"/>
+      <c r="F38" s="17"/>
+      <c r="G38" s="17"/>
+    </row>
+    <row r="39" ht="28" customHeight="1" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B39" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="C39" s="17"/>
+      <c r="D39" s="17"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
+      <c r="G39" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B29:G29"/>
-    <mergeCell ref="B30:G30"/>
-    <mergeCell ref="B31:G31"/>
-    <mergeCell ref="B32:G32"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B39:G39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -3318,7 +3702,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:L80"/>
+  <dimension ref="B2:L87"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
@@ -3337,7 +3721,7 @@
   <sheetData>
     <row r="2" ht="36" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B2" s="18" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -3352,2697 +3736,2942 @@
     </row>
     <row r="4" ht="28" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B4" s="19" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="I4" s="20" t="s">
-        <v>72</v>
+        <v>87</v>
       </c>
       <c r="J4" s="19" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="L4" s="20" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B5" s="21" t="s">
-        <v>76</v>
+        <v>91</v>
       </c>
       <c r="C5" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D5" s="22" t="s">
-        <v>77</v>
+        <v>92</v>
       </c>
       <c r="E5" s="22" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="G5" s="22" t="s">
-        <v>80</v>
+        <v>95</v>
       </c>
       <c r="H5" s="22" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="I5" s="22" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="J5" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K5" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L5" s="22" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B6" s="21" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="C6" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D6" s="22" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="F6" s="22" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>88</v>
+        <v>103</v>
       </c>
       <c r="H6" s="22" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="I6" s="22" t="s">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="J6" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K6" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L6" s="22" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B7" s="21" t="s">
-        <v>92</v>
+        <v>107</v>
       </c>
       <c r="C7" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>93</v>
+        <v>108</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="G7" s="22" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="H7" s="22" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="I7" s="22" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K7" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L7" s="22" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B8" s="21" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="C8" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>101</v>
+        <v>116</v>
       </c>
       <c r="E8" s="22" t="s">
-        <v>102</v>
+        <v>117</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="G8" s="22" t="s">
-        <v>104</v>
+        <v>119</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>105</v>
+        <v>120</v>
       </c>
       <c r="I8" s="22" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K8" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L8" s="22" t="s">
-        <v>107</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B9" s="21" t="s">
-        <v>108</v>
+        <v>123</v>
       </c>
       <c r="C9" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>112</v>
+        <v>127</v>
       </c>
       <c r="H9" s="22" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="I9" s="22" t="s">
-        <v>114</v>
+        <v>129</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K9" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L9" s="22" t="s">
-        <v>115</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B10" s="21" t="s">
-        <v>116</v>
+        <v>131</v>
       </c>
       <c r="C10" s="22" t="s">
         <v>18</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>117</v>
+        <v>132</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
       <c r="F10" s="22" t="s">
-        <v>118</v>
+        <v>133</v>
       </c>
       <c r="G10" s="22" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="H10" s="22" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
       <c r="I10" s="22" t="s">
-        <v>121</v>
+        <v>136</v>
       </c>
       <c r="J10" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K10" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L10" s="22" t="s">
-        <v>122</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B11" s="21" t="s">
-        <v>123</v>
+        <v>138</v>
       </c>
       <c r="C11" s="22" t="s">
         <v>23</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>124</v>
+        <v>139</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>126</v>
+        <v>141</v>
       </c>
       <c r="G11" s="22" t="s">
-        <v>127</v>
+        <v>142</v>
       </c>
       <c r="H11" s="22" t="s">
-        <v>128</v>
+        <v>143</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="J11" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K11" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L11" s="22" t="s">
-        <v>130</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B12" s="21" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="C12" s="22" t="s">
         <v>23</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>132</v>
+        <v>147</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="F12" s="22" t="s">
-        <v>133</v>
+        <v>148</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="H12" s="22" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="I12" s="22" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K12" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L12" s="22" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B13" s="21" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="C13" s="22" t="s">
         <v>23</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="F13" s="22" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="G13" s="22" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="H13" s="22" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="I13" s="22" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K13" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L13" s="22" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B14" s="21" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="C14" s="22" t="s">
         <v>26</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="F14" s="22" t="s">
-        <v>149</v>
+        <v>164</v>
       </c>
       <c r="G14" s="22" t="s">
-        <v>150</v>
+        <v>165</v>
       </c>
       <c r="H14" s="22" t="s">
-        <v>151</v>
+        <v>166</v>
       </c>
       <c r="I14" s="22" t="s">
-        <v>152</v>
+        <v>167</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K14" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L14" s="22" t="s">
-        <v>153</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B15" s="21" t="s">
-        <v>154</v>
+        <v>169</v>
       </c>
       <c r="C15" s="22" t="s">
         <v>26</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="F15" s="22" t="s">
-        <v>111</v>
+        <v>126</v>
       </c>
       <c r="G15" s="22" t="s">
-        <v>156</v>
+        <v>171</v>
       </c>
       <c r="H15" s="22" t="s">
-        <v>157</v>
+        <v>172</v>
       </c>
       <c r="I15" s="22" t="s">
-        <v>158</v>
+        <v>173</v>
       </c>
       <c r="J15" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K15" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L15" s="22" t="s">
-        <v>159</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B16" s="21" t="s">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="C16" s="22" t="s">
         <v>26</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>161</v>
+        <v>176</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>162</v>
+        <v>177</v>
       </c>
       <c r="F16" s="22" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="G16" s="22" t="s">
-        <v>164</v>
+        <v>179</v>
       </c>
       <c r="H16" s="22" t="s">
-        <v>165</v>
+        <v>180</v>
       </c>
       <c r="I16" s="22" t="s">
-        <v>166</v>
+        <v>181</v>
       </c>
       <c r="J16" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K16" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L16" s="22" t="s">
-        <v>167</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="21" t="s">
-        <v>168</v>
+        <v>183</v>
       </c>
       <c r="C17" s="22" t="s">
         <v>29</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>169</v>
+        <v>184</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F17" s="22" t="s">
-        <v>171</v>
+        <v>186</v>
       </c>
       <c r="G17" s="22" t="s">
-        <v>172</v>
+        <v>187</v>
       </c>
       <c r="H17" s="22" t="s">
-        <v>173</v>
+        <v>188</v>
       </c>
       <c r="I17" s="22" t="s">
-        <v>174</v>
+        <v>189</v>
       </c>
       <c r="J17" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K17" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L17" s="22" t="s">
-        <v>175</v>
+        <v>190</v>
       </c>
     </row>
     <row r="18" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="21" t="s">
-        <v>176</v>
+        <v>191</v>
       </c>
       <c r="C18" s="22" t="s">
         <v>29</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>178</v>
+        <v>193</v>
       </c>
       <c r="F18" s="22" t="s">
-        <v>179</v>
+        <v>194</v>
       </c>
       <c r="G18" s="22" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="H18" s="22" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="I18" s="22" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="J18" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K18" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L18" s="22" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
     </row>
     <row r="19" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="21" t="s">
-        <v>184</v>
+        <v>199</v>
       </c>
       <c r="C19" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>185</v>
+        <v>200</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>186</v>
+        <v>201</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="G19" s="22" t="s">
-        <v>188</v>
+        <v>203</v>
       </c>
       <c r="H19" s="22" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="I19" s="22" t="s">
-        <v>190</v>
+        <v>205</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K19" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L19" s="22" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
     </row>
     <row r="20" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="21" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="C20" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="G20" s="22" t="s">
-        <v>196</v>
+        <v>211</v>
       </c>
       <c r="H20" s="22" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="I20" s="22" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K20" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L20" s="22" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
     </row>
     <row r="21" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="21" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C21" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>201</v>
+        <v>216</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>202</v>
+        <v>217</v>
       </c>
       <c r="F21" s="22" t="s">
-        <v>203</v>
+        <v>218</v>
       </c>
       <c r="G21" s="22" t="s">
-        <v>204</v>
+        <v>219</v>
       </c>
       <c r="H21" s="22" t="s">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="I21" s="22" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
       <c r="J21" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K21" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L21" s="22" t="s">
-        <v>207</v>
+        <v>222</v>
       </c>
     </row>
     <row r="22" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="21" t="s">
-        <v>208</v>
+        <v>223</v>
       </c>
       <c r="C22" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>209</v>
+        <v>224</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>210</v>
+        <v>225</v>
       </c>
       <c r="F22" s="22" t="s">
-        <v>211</v>
+        <v>226</v>
       </c>
       <c r="G22" s="22" t="s">
-        <v>212</v>
+        <v>227</v>
       </c>
       <c r="H22" s="22" t="s">
-        <v>213</v>
+        <v>228</v>
       </c>
       <c r="I22" s="22" t="s">
-        <v>214</v>
+        <v>229</v>
       </c>
       <c r="J22" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K22" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L22" s="22" t="s">
-        <v>215</v>
+        <v>230</v>
       </c>
     </row>
     <row r="23" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="21" t="s">
-        <v>216</v>
+        <v>231</v>
       </c>
       <c r="C23" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
       <c r="F23" s="22" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="H23" s="22" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
       <c r="I23" s="22" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
       <c r="J23" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K23" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L23" s="22" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
     </row>
     <row r="24" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="21" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="C24" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>225</v>
+        <v>240</v>
       </c>
       <c r="E24" s="22" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="F24" s="22" t="s">
-        <v>227</v>
+        <v>242</v>
       </c>
       <c r="G24" s="22" t="s">
-        <v>228</v>
+        <v>243</v>
       </c>
       <c r="H24" s="22" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
       <c r="I24" s="22" t="s">
-        <v>230</v>
+        <v>245</v>
       </c>
       <c r="J24" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K24" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L24" s="22" t="s">
-        <v>231</v>
+        <v>246</v>
       </c>
     </row>
     <row r="25" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="21" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
       <c r="C25" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="E25" s="22" t="s">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="F25" s="22" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="G25" s="22" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="H25" s="22" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
       <c r="I25" s="22" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
       <c r="J25" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K25" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L25" s="22" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
     </row>
     <row r="26" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="21" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="C26" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D26" s="22" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="E26" s="22" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="F26" s="22" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="G26" s="22" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="H26" s="22" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="I26" s="22" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="J26" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K26" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L26" s="22" t="s">
-        <v>246</v>
+        <v>261</v>
       </c>
     </row>
     <row r="27" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="21" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="C27" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="E27" s="22" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="F27" s="22" t="s">
-        <v>249</v>
+        <v>264</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="H27" s="22" t="s">
-        <v>251</v>
+        <v>266</v>
       </c>
       <c r="I27" s="22" t="s">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="J27" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K27" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L27" s="22" t="s">
-        <v>253</v>
+        <v>268</v>
       </c>
     </row>
     <row r="28" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" s="21" t="s">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="C28" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D28" s="22" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="F28" s="22" t="s">
-        <v>257</v>
+        <v>272</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>258</v>
+        <v>273</v>
       </c>
       <c r="H28" s="22" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
       <c r="I28" s="22" t="s">
-        <v>260</v>
+        <v>275</v>
       </c>
       <c r="J28" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K28" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L28" s="22" t="s">
-        <v>261</v>
+        <v>276</v>
       </c>
     </row>
     <row r="29" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" s="21" t="s">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="C29" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D29" s="22" t="s">
-        <v>263</v>
+        <v>278</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>264</v>
+        <v>279</v>
       </c>
       <c r="F29" s="22" t="s">
-        <v>265</v>
+        <v>280</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>266</v>
+        <v>281</v>
       </c>
       <c r="H29" s="22" t="s">
-        <v>267</v>
+        <v>282</v>
       </c>
       <c r="I29" s="22" t="s">
-        <v>268</v>
+        <v>283</v>
       </c>
       <c r="J29" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K29" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L29" s="22" t="s">
-        <v>269</v>
+        <v>284</v>
       </c>
     </row>
     <row r="30" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="21" t="s">
-        <v>270</v>
+        <v>285</v>
       </c>
       <c r="C30" s="22" t="s">
         <v>37</v>
       </c>
       <c r="D30" s="22" t="s">
-        <v>271</v>
+        <v>286</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>272</v>
+        <v>287</v>
       </c>
       <c r="F30" s="22" t="s">
-        <v>273</v>
+        <v>288</v>
       </c>
       <c r="G30" s="22" t="s">
-        <v>274</v>
+        <v>289</v>
       </c>
       <c r="H30" s="22" t="s">
-        <v>275</v>
+        <v>290</v>
       </c>
       <c r="I30" s="22" t="s">
-        <v>276</v>
+        <v>291</v>
       </c>
       <c r="J30" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K30" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L30" s="22" t="s">
-        <v>277</v>
+        <v>292</v>
       </c>
     </row>
     <row r="31" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B31" s="21" t="s">
-        <v>278</v>
+        <v>293</v>
       </c>
       <c r="C31" s="22" t="s">
         <v>37</v>
       </c>
       <c r="D31" s="22" t="s">
-        <v>279</v>
+        <v>294</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>280</v>
+        <v>295</v>
       </c>
       <c r="F31" s="22" t="s">
-        <v>281</v>
+        <v>296</v>
       </c>
       <c r="G31" s="22" t="s">
-        <v>282</v>
+        <v>297</v>
       </c>
       <c r="H31" s="22" t="s">
-        <v>283</v>
+        <v>298</v>
       </c>
       <c r="I31" s="22" t="s">
-        <v>284</v>
+        <v>299</v>
       </c>
       <c r="J31" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K31" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L31" s="22" t="s">
-        <v>285</v>
+        <v>300</v>
       </c>
     </row>
     <row r="32" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B32" s="21" t="s">
-        <v>286</v>
+        <v>301</v>
       </c>
       <c r="C32" s="22" t="s">
         <v>39</v>
       </c>
       <c r="D32" s="22" t="s">
-        <v>287</v>
+        <v>302</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>288</v>
+        <v>303</v>
       </c>
       <c r="F32" s="22" t="s">
-        <v>289</v>
+        <v>304</v>
       </c>
       <c r="G32" s="22" t="s">
-        <v>290</v>
+        <v>305</v>
       </c>
       <c r="H32" s="22" t="s">
-        <v>291</v>
+        <v>306</v>
       </c>
       <c r="I32" s="22" t="s">
-        <v>292</v>
+        <v>307</v>
       </c>
       <c r="J32" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K32" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L32" s="22" t="s">
-        <v>293</v>
+        <v>308</v>
       </c>
     </row>
     <row r="33" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B33" s="21" t="s">
-        <v>294</v>
+        <v>309</v>
       </c>
       <c r="C33" s="22" t="s">
         <v>39</v>
       </c>
       <c r="D33" s="22" t="s">
-        <v>295</v>
+        <v>310</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>288</v>
+        <v>303</v>
       </c>
       <c r="F33" s="22" t="s">
-        <v>296</v>
+        <v>311</v>
       </c>
       <c r="G33" s="22" t="s">
-        <v>297</v>
+        <v>312</v>
       </c>
       <c r="H33" s="22" t="s">
-        <v>298</v>
+        <v>313</v>
       </c>
       <c r="I33" s="22" t="s">
-        <v>299</v>
+        <v>314</v>
       </c>
       <c r="J33" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K33" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L33" s="22" t="s">
-        <v>300</v>
+        <v>315</v>
       </c>
     </row>
     <row r="34" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B34" s="21" t="s">
-        <v>301</v>
+        <v>316</v>
       </c>
       <c r="C34" s="22" t="s">
         <v>39</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>302</v>
+        <v>317</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>288</v>
+        <v>303</v>
       </c>
       <c r="F34" s="22" t="s">
-        <v>303</v>
+        <v>318</v>
       </c>
       <c r="G34" s="22" t="s">
-        <v>304</v>
+        <v>319</v>
       </c>
       <c r="H34" s="22" t="s">
-        <v>305</v>
+        <v>320</v>
       </c>
       <c r="I34" s="22" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="J34" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K34" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L34" s="22" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
     </row>
     <row r="35" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B35" s="21" t="s">
-        <v>308</v>
+        <v>323</v>
       </c>
       <c r="C35" s="22" t="s">
         <v>41</v>
       </c>
       <c r="D35" s="22" t="s">
-        <v>309</v>
+        <v>324</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="F35" s="22" t="s">
-        <v>311</v>
+        <v>326</v>
       </c>
       <c r="G35" s="22" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="H35" s="22" t="s">
-        <v>313</v>
+        <v>328</v>
       </c>
       <c r="I35" s="22" t="s">
-        <v>314</v>
+        <v>329</v>
       </c>
       <c r="J35" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K35" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L35" s="22" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
     </row>
     <row r="36" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B36" s="21" t="s">
-        <v>316</v>
+        <v>331</v>
       </c>
       <c r="C36" s="22" t="s">
         <v>41</v>
       </c>
       <c r="D36" s="22" t="s">
-        <v>317</v>
+        <v>332</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>318</v>
+        <v>333</v>
       </c>
       <c r="F36" s="22" t="s">
-        <v>319</v>
+        <v>334</v>
       </c>
       <c r="G36" s="22" t="s">
-        <v>320</v>
+        <v>335</v>
       </c>
       <c r="H36" s="22" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
       <c r="I36" s="22" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="J36" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K36" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L36" s="22" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
     </row>
     <row r="37" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B37" s="21" t="s">
-        <v>324</v>
+        <v>339</v>
       </c>
       <c r="C37" s="22" t="s">
         <v>41</v>
       </c>
       <c r="D37" s="22" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>326</v>
+        <v>341</v>
       </c>
       <c r="F37" s="22" t="s">
-        <v>327</v>
+        <v>342</v>
       </c>
       <c r="G37" s="22" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="H37" s="22" t="s">
-        <v>329</v>
+        <v>344</v>
       </c>
       <c r="I37" s="22" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="J37" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K37" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L37" s="22" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
     </row>
     <row r="38" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B38" s="21" t="s">
-        <v>332</v>
+        <v>347</v>
       </c>
       <c r="C38" s="22" t="s">
         <v>41</v>
       </c>
       <c r="D38" s="22" t="s">
-        <v>333</v>
+        <v>348</v>
       </c>
       <c r="E38" s="22" t="s">
-        <v>334</v>
+        <v>349</v>
       </c>
       <c r="F38" s="22" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
       <c r="G38" s="22" t="s">
-        <v>336</v>
+        <v>351</v>
       </c>
       <c r="H38" s="22" t="s">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="I38" s="22" t="s">
-        <v>338</v>
+        <v>353</v>
       </c>
       <c r="J38" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K38" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L38" s="22" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
     </row>
     <row r="39" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B39" s="21" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
       <c r="C39" s="22" t="s">
         <v>44</v>
       </c>
       <c r="D39" s="22" t="s">
-        <v>341</v>
+        <v>356</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
       <c r="F39" s="22" t="s">
-        <v>227</v>
+        <v>242</v>
       </c>
       <c r="G39" s="22" t="s">
-        <v>343</v>
+        <v>358</v>
       </c>
       <c r="H39" s="22" t="s">
-        <v>344</v>
+        <v>359</v>
       </c>
       <c r="I39" s="22" t="s">
-        <v>345</v>
+        <v>360</v>
       </c>
       <c r="J39" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K39" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L39" s="22" t="s">
-        <v>346</v>
+        <v>361</v>
       </c>
     </row>
     <row r="40" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B40" s="21" t="s">
-        <v>347</v>
+        <v>362</v>
       </c>
       <c r="C40" s="22" t="s">
         <v>44</v>
       </c>
       <c r="D40" s="22" t="s">
-        <v>348</v>
+        <v>363</v>
       </c>
       <c r="E40" s="22" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
       <c r="F40" s="22" t="s">
-        <v>349</v>
+        <v>364</v>
       </c>
       <c r="G40" s="22" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="H40" s="22" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
       <c r="I40" s="22" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="J40" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K40" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L40" s="22" t="s">
-        <v>353</v>
+        <v>368</v>
       </c>
     </row>
     <row r="41" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B41" s="21" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
       <c r="C41" s="22" t="s">
         <v>46</v>
       </c>
       <c r="D41" s="22" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="E41" s="22" t="s">
-        <v>356</v>
+        <v>371</v>
       </c>
       <c r="F41" s="22" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
       <c r="G41" s="22" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="H41" s="22" t="s">
-        <v>359</v>
+        <v>374</v>
       </c>
       <c r="I41" s="22" t="s">
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="J41" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K41" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L41" s="22" t="s">
-        <v>361</v>
+        <v>376</v>
       </c>
     </row>
     <row r="42" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B42" s="21" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
       <c r="C42" s="22" t="s">
         <v>46</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>363</v>
+        <v>378</v>
       </c>
       <c r="E42" s="22" t="s">
-        <v>364</v>
+        <v>379</v>
       </c>
       <c r="F42" s="22" t="s">
-        <v>365</v>
+        <v>380</v>
       </c>
       <c r="G42" s="22" t="s">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="H42" s="22" t="s">
-        <v>367</v>
+        <v>382</v>
       </c>
       <c r="I42" s="22" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
       <c r="J42" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K42" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L42" s="22" t="s">
-        <v>369</v>
+        <v>384</v>
       </c>
     </row>
     <row r="43" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B43" s="21" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
       <c r="C43" s="22" t="s">
         <v>48</v>
       </c>
       <c r="D43" s="22" t="s">
-        <v>371</v>
+        <v>386</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
       <c r="F43" s="22" t="s">
-        <v>373</v>
+        <v>388</v>
       </c>
       <c r="G43" s="22" t="s">
-        <v>374</v>
+        <v>389</v>
       </c>
       <c r="H43" s="22" t="s">
-        <v>375</v>
+        <v>390</v>
       </c>
       <c r="I43" s="22" t="s">
-        <v>376</v>
+        <v>391</v>
       </c>
       <c r="J43" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K43" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L43" s="22" t="s">
-        <v>377</v>
+        <v>392</v>
       </c>
     </row>
     <row r="44" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B44" s="21" t="s">
-        <v>378</v>
+        <v>393</v>
       </c>
       <c r="C44" s="22" t="s">
         <v>48</v>
       </c>
       <c r="D44" s="22" t="s">
-        <v>379</v>
+        <v>394</v>
       </c>
       <c r="E44" s="22" t="s">
-        <v>380</v>
+        <v>395</v>
       </c>
       <c r="F44" s="22" t="s">
-        <v>381</v>
+        <v>396</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>382</v>
+        <v>397</v>
       </c>
       <c r="H44" s="22" t="s">
-        <v>383</v>
+        <v>398</v>
       </c>
       <c r="I44" s="22" t="s">
-        <v>384</v>
+        <v>399</v>
       </c>
       <c r="J44" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K44" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L44" s="22" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
     </row>
     <row r="45" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B45" s="21" t="s">
-        <v>386</v>
+        <v>401</v>
       </c>
       <c r="C45" s="22" t="s">
         <v>48</v>
       </c>
       <c r="D45" s="22" t="s">
-        <v>387</v>
+        <v>402</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>388</v>
+        <v>403</v>
       </c>
       <c r="F45" s="22" t="s">
-        <v>389</v>
+        <v>404</v>
       </c>
       <c r="G45" s="22" t="s">
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="H45" s="22" t="s">
-        <v>391</v>
+        <v>406</v>
       </c>
       <c r="I45" s="22" t="s">
-        <v>392</v>
+        <v>407</v>
       </c>
       <c r="J45" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K45" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L45" s="22" t="s">
-        <v>393</v>
+        <v>408</v>
       </c>
     </row>
     <row r="46" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B46" s="21" t="s">
-        <v>394</v>
+        <v>409</v>
       </c>
       <c r="C46" s="22" t="s">
         <v>48</v>
       </c>
       <c r="D46" s="22" t="s">
-        <v>395</v>
+        <v>410</v>
       </c>
       <c r="E46" s="22" t="s">
-        <v>396</v>
+        <v>411</v>
       </c>
       <c r="F46" s="22" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="G46" s="22" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="H46" s="22" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="I46" s="22" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="J46" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K46" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L46" s="22" t="s">
-        <v>401</v>
+        <v>416</v>
       </c>
     </row>
     <row r="47" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B47" s="21" t="s">
-        <v>402</v>
+        <v>417</v>
       </c>
       <c r="C47" s="22" t="s">
         <v>48</v>
       </c>
       <c r="D47" s="22" t="s">
-        <v>403</v>
+        <v>418</v>
       </c>
       <c r="E47" s="22" t="s">
-        <v>404</v>
+        <v>419</v>
       </c>
       <c r="F47" s="22" t="s">
-        <v>405</v>
+        <v>420</v>
       </c>
       <c r="G47" s="22" t="s">
-        <v>406</v>
+        <v>421</v>
       </c>
       <c r="H47" s="22" t="s">
-        <v>407</v>
+        <v>422</v>
       </c>
       <c r="I47" s="22" t="s">
-        <v>408</v>
+        <v>423</v>
       </c>
       <c r="J47" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K47" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L47" s="22" t="s">
-        <v>409</v>
+        <v>424</v>
       </c>
     </row>
     <row r="48" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48" s="21" t="s">
-        <v>410</v>
+        <v>425</v>
       </c>
       <c r="C48" s="22" t="s">
         <v>48</v>
       </c>
       <c r="D48" s="22" t="s">
-        <v>411</v>
+        <v>426</v>
       </c>
       <c r="E48" s="22" t="s">
-        <v>412</v>
+        <v>427</v>
       </c>
       <c r="F48" s="22" t="s">
-        <v>413</v>
+        <v>428</v>
       </c>
       <c r="G48" s="22" t="s">
-        <v>414</v>
+        <v>429</v>
       </c>
       <c r="H48" s="22" t="s">
-        <v>415</v>
+        <v>430</v>
       </c>
       <c r="I48" s="22" t="s">
-        <v>416</v>
+        <v>431</v>
       </c>
       <c r="J48" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K48" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L48" s="22" t="s">
-        <v>417</v>
+        <v>432</v>
       </c>
     </row>
     <row r="49" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B49" s="21" t="s">
-        <v>418</v>
+        <v>433</v>
       </c>
       <c r="C49" s="22" t="s">
         <v>48</v>
       </c>
       <c r="D49" s="22" t="s">
-        <v>419</v>
+        <v>434</v>
       </c>
       <c r="E49" s="22" t="s">
-        <v>420</v>
+        <v>435</v>
       </c>
       <c r="F49" s="22" t="s">
-        <v>421</v>
+        <v>436</v>
       </c>
       <c r="G49" s="22" t="s">
-        <v>422</v>
+        <v>437</v>
       </c>
       <c r="H49" s="22" t="s">
-        <v>423</v>
+        <v>438</v>
       </c>
       <c r="I49" s="22" t="s">
-        <v>424</v>
+        <v>439</v>
       </c>
       <c r="J49" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K49" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L49" s="22" t="s">
-        <v>425</v>
+        <v>440</v>
       </c>
     </row>
     <row r="50" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B50" s="21" t="s">
-        <v>426</v>
+        <v>441</v>
       </c>
       <c r="C50" s="22" t="s">
         <v>48</v>
       </c>
       <c r="D50" s="22" t="s">
-        <v>427</v>
+        <v>442</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>396</v>
+        <v>411</v>
       </c>
       <c r="F50" s="22" t="s">
-        <v>428</v>
+        <v>443</v>
       </c>
       <c r="G50" s="22" t="s">
-        <v>429</v>
+        <v>444</v>
       </c>
       <c r="H50" s="22" t="s">
-        <v>430</v>
+        <v>445</v>
       </c>
       <c r="I50" s="22" t="s">
-        <v>431</v>
+        <v>446</v>
       </c>
       <c r="J50" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K50" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L50" s="22" t="s">
-        <v>432</v>
+        <v>447</v>
       </c>
     </row>
     <row r="51" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B51" s="21" t="s">
-        <v>433</v>
+        <v>448</v>
       </c>
       <c r="C51" s="22" t="s">
         <v>48</v>
       </c>
       <c r="D51" s="22" t="s">
-        <v>434</v>
+        <v>449</v>
       </c>
       <c r="E51" s="22" t="s">
-        <v>435</v>
+        <v>450</v>
       </c>
       <c r="F51" s="22" t="s">
-        <v>436</v>
+        <v>451</v>
       </c>
       <c r="G51" s="22" t="s">
-        <v>437</v>
+        <v>452</v>
       </c>
       <c r="H51" s="22" t="s">
-        <v>438</v>
+        <v>453</v>
       </c>
       <c r="I51" s="22" t="s">
-        <v>439</v>
+        <v>454</v>
       </c>
       <c r="J51" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K51" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L51" s="22" t="s">
-        <v>440</v>
+        <v>455</v>
       </c>
     </row>
     <row r="52" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B52" s="21" t="s">
-        <v>441</v>
+        <v>456</v>
       </c>
       <c r="C52" s="22" t="s">
         <v>51</v>
       </c>
       <c r="D52" s="22" t="s">
-        <v>442</v>
+        <v>457</v>
       </c>
       <c r="E52" s="22" t="s">
-        <v>443</v>
+        <v>458</v>
       </c>
       <c r="F52" s="22" t="s">
-        <v>444</v>
+        <v>459</v>
       </c>
       <c r="G52" s="22" t="s">
-        <v>445</v>
+        <v>460</v>
       </c>
       <c r="H52" s="22" t="s">
-        <v>446</v>
+        <v>461</v>
       </c>
       <c r="I52" s="22" t="s">
-        <v>447</v>
+        <v>462</v>
       </c>
       <c r="J52" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K52" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L52" s="22" t="s">
-        <v>448</v>
+        <v>463</v>
       </c>
     </row>
     <row r="53" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B53" s="21" t="s">
-        <v>449</v>
+        <v>464</v>
       </c>
       <c r="C53" s="22" t="s">
         <v>51</v>
       </c>
       <c r="D53" s="22" t="s">
-        <v>450</v>
+        <v>465</v>
       </c>
       <c r="E53" s="22" t="s">
-        <v>443</v>
+        <v>458</v>
       </c>
       <c r="F53" s="22" t="s">
-        <v>451</v>
+        <v>466</v>
       </c>
       <c r="G53" s="22" t="s">
-        <v>452</v>
+        <v>467</v>
       </c>
       <c r="H53" s="22" t="s">
-        <v>453</v>
+        <v>468</v>
       </c>
       <c r="I53" s="22" t="s">
-        <v>454</v>
+        <v>469</v>
       </c>
       <c r="J53" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K53" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L53" s="22" t="s">
-        <v>455</v>
+        <v>470</v>
       </c>
     </row>
     <row r="54" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B54" s="21" t="s">
-        <v>456</v>
+        <v>471</v>
       </c>
       <c r="C54" s="22" t="s">
         <v>53</v>
       </c>
       <c r="D54" s="22" t="s">
-        <v>457</v>
+        <v>472</v>
       </c>
       <c r="E54" s="22" t="s">
-        <v>458</v>
+        <v>473</v>
       </c>
       <c r="F54" s="22" t="s">
-        <v>227</v>
+        <v>242</v>
       </c>
       <c r="G54" s="22" t="s">
-        <v>459</v>
+        <v>474</v>
       </c>
       <c r="H54" s="22" t="s">
-        <v>460</v>
+        <v>475</v>
       </c>
       <c r="I54" s="22" t="s">
-        <v>461</v>
+        <v>476</v>
       </c>
       <c r="J54" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K54" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L54" s="22" t="s">
-        <v>462</v>
+        <v>477</v>
       </c>
     </row>
     <row r="55" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B55" s="21" t="s">
-        <v>463</v>
+        <v>478</v>
       </c>
       <c r="C55" s="22" t="s">
         <v>53</v>
       </c>
       <c r="D55" s="22" t="s">
-        <v>464</v>
+        <v>479</v>
       </c>
       <c r="E55" s="22" t="s">
-        <v>465</v>
+        <v>480</v>
       </c>
       <c r="F55" s="22" t="s">
-        <v>466</v>
+        <v>481</v>
       </c>
       <c r="G55" s="22" t="s">
-        <v>467</v>
+        <v>482</v>
       </c>
       <c r="H55" s="22" t="s">
-        <v>468</v>
+        <v>483</v>
       </c>
       <c r="I55" s="22" t="s">
-        <v>469</v>
+        <v>484</v>
       </c>
       <c r="J55" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K55" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L55" s="22" t="s">
-        <v>470</v>
+        <v>485</v>
       </c>
     </row>
     <row r="56" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B56" s="21" t="s">
-        <v>471</v>
+        <v>486</v>
       </c>
       <c r="C56" s="22" t="s">
         <v>53</v>
       </c>
       <c r="D56" s="22" t="s">
-        <v>472</v>
+        <v>487</v>
       </c>
       <c r="E56" s="22" t="s">
-        <v>465</v>
+        <v>480</v>
       </c>
       <c r="F56" s="22" t="s">
-        <v>473</v>
+        <v>488</v>
       </c>
       <c r="G56" s="22" t="s">
-        <v>474</v>
+        <v>489</v>
       </c>
       <c r="H56" s="22" t="s">
-        <v>475</v>
+        <v>490</v>
       </c>
       <c r="I56" s="22" t="s">
-        <v>476</v>
+        <v>491</v>
       </c>
       <c r="J56" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K56" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L56" s="22" t="s">
-        <v>477</v>
+        <v>492</v>
       </c>
     </row>
     <row r="57" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B57" s="21" t="s">
-        <v>478</v>
+        <v>493</v>
       </c>
       <c r="C57" s="22" t="s">
         <v>55</v>
       </c>
       <c r="D57" s="22" t="s">
-        <v>479</v>
+        <v>494</v>
       </c>
       <c r="E57" s="22" t="s">
-        <v>480</v>
+        <v>495</v>
       </c>
       <c r="F57" s="22" t="s">
-        <v>481</v>
+        <v>496</v>
       </c>
       <c r="G57" s="22" t="s">
-        <v>482</v>
+        <v>497</v>
       </c>
       <c r="H57" s="22" t="s">
-        <v>483</v>
+        <v>498</v>
       </c>
       <c r="I57" s="22" t="s">
-        <v>484</v>
+        <v>499</v>
       </c>
       <c r="J57" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K57" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L57" s="22" t="s">
-        <v>485</v>
+        <v>500</v>
       </c>
     </row>
     <row r="58" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B58" s="21" t="s">
-        <v>486</v>
+        <v>501</v>
       </c>
       <c r="C58" s="22" t="s">
         <v>55</v>
       </c>
       <c r="D58" s="22" t="s">
-        <v>487</v>
+        <v>502</v>
       </c>
       <c r="E58" s="22" t="s">
-        <v>488</v>
+        <v>503</v>
       </c>
       <c r="F58" s="22" t="s">
-        <v>489</v>
+        <v>504</v>
       </c>
       <c r="G58" s="22" t="s">
-        <v>490</v>
+        <v>505</v>
       </c>
       <c r="H58" s="22" t="s">
-        <v>491</v>
+        <v>506</v>
       </c>
       <c r="I58" s="22" t="s">
-        <v>492</v>
+        <v>507</v>
       </c>
       <c r="J58" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K58" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L58" s="22" t="s">
-        <v>493</v>
+        <v>508</v>
       </c>
     </row>
     <row r="59" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B59" s="21" t="s">
-        <v>494</v>
+        <v>509</v>
       </c>
       <c r="C59" s="22" t="s">
         <v>55</v>
       </c>
       <c r="D59" s="22" t="s">
-        <v>495</v>
+        <v>510</v>
       </c>
       <c r="E59" s="22" t="s">
-        <v>496</v>
+        <v>511</v>
       </c>
       <c r="F59" s="22" t="s">
-        <v>497</v>
+        <v>512</v>
       </c>
       <c r="G59" s="22" t="s">
-        <v>498</v>
+        <v>513</v>
       </c>
       <c r="H59" s="22" t="s">
-        <v>499</v>
+        <v>514</v>
       </c>
       <c r="I59" s="22" t="s">
-        <v>500</v>
+        <v>515</v>
       </c>
       <c r="J59" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K59" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L59" s="22" t="s">
-        <v>501</v>
+        <v>516</v>
       </c>
     </row>
     <row r="60" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B60" s="21" t="s">
-        <v>502</v>
+        <v>517</v>
       </c>
       <c r="C60" s="22" t="s">
         <v>55</v>
       </c>
       <c r="D60" s="22" t="s">
-        <v>503</v>
+        <v>518</v>
       </c>
       <c r="E60" s="22" t="s">
-        <v>504</v>
+        <v>519</v>
       </c>
       <c r="F60" s="22" t="s">
-        <v>505</v>
+        <v>520</v>
       </c>
       <c r="G60" s="22" t="s">
-        <v>506</v>
+        <v>521</v>
       </c>
       <c r="H60" s="22" t="s">
-        <v>507</v>
+        <v>522</v>
       </c>
       <c r="I60" s="22" t="s">
-        <v>508</v>
+        <v>523</v>
       </c>
       <c r="J60" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K60" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L60" s="22" t="s">
-        <v>509</v>
+        <v>524</v>
       </c>
     </row>
     <row r="61" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B61" s="21" t="s">
-        <v>510</v>
+        <v>525</v>
       </c>
       <c r="C61" s="22" t="s">
         <v>57</v>
       </c>
       <c r="D61" s="22" t="s">
-        <v>511</v>
+        <v>526</v>
       </c>
       <c r="E61" s="22" t="s">
-        <v>512</v>
+        <v>527</v>
       </c>
       <c r="F61" s="22" t="s">
-        <v>513</v>
+        <v>528</v>
       </c>
       <c r="G61" s="22" t="s">
-        <v>514</v>
+        <v>529</v>
       </c>
       <c r="H61" s="22" t="s">
-        <v>515</v>
+        <v>530</v>
       </c>
       <c r="I61" s="22" t="s">
-        <v>516</v>
+        <v>531</v>
       </c>
       <c r="J61" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K61" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L61" s="22" t="s">
-        <v>517</v>
+        <v>532</v>
       </c>
     </row>
     <row r="62" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B62" s="21" t="s">
-        <v>518</v>
+        <v>533</v>
       </c>
       <c r="C62" s="22" t="s">
         <v>57</v>
       </c>
       <c r="D62" s="22" t="s">
-        <v>519</v>
+        <v>534</v>
       </c>
       <c r="E62" s="22" t="s">
-        <v>520</v>
+        <v>535</v>
       </c>
       <c r="F62" s="22" t="s">
-        <v>521</v>
+        <v>536</v>
       </c>
       <c r="G62" s="22" t="s">
-        <v>522</v>
+        <v>537</v>
       </c>
       <c r="H62" s="22" t="s">
-        <v>523</v>
+        <v>538</v>
       </c>
       <c r="I62" s="22" t="s">
-        <v>524</v>
+        <v>539</v>
       </c>
       <c r="J62" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K62" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L62" s="22" t="s">
-        <v>525</v>
+        <v>540</v>
       </c>
     </row>
     <row r="63" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B63" s="21" t="s">
-        <v>526</v>
+        <v>541</v>
       </c>
       <c r="C63" s="22" t="s">
         <v>57</v>
       </c>
       <c r="D63" s="22" t="s">
-        <v>527</v>
+        <v>542</v>
       </c>
       <c r="E63" s="22" t="s">
-        <v>528</v>
+        <v>543</v>
       </c>
       <c r="F63" s="22" t="s">
-        <v>529</v>
+        <v>544</v>
       </c>
       <c r="G63" s="22" t="s">
-        <v>530</v>
+        <v>545</v>
       </c>
       <c r="H63" s="22" t="s">
-        <v>531</v>
+        <v>546</v>
       </c>
       <c r="I63" s="22" t="s">
-        <v>532</v>
+        <v>547</v>
       </c>
       <c r="J63" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K63" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L63" s="22" t="s">
-        <v>533</v>
+        <v>548</v>
       </c>
     </row>
     <row r="64" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B64" s="21" t="s">
-        <v>534</v>
+        <v>549</v>
       </c>
       <c r="C64" s="22" t="s">
         <v>59</v>
       </c>
       <c r="D64" s="22" t="s">
-        <v>535</v>
+        <v>550</v>
       </c>
       <c r="E64" s="22" t="s">
-        <v>536</v>
+        <v>551</v>
       </c>
       <c r="F64" s="22" t="s">
-        <v>537</v>
+        <v>552</v>
       </c>
       <c r="G64" s="22" t="s">
-        <v>538</v>
+        <v>553</v>
       </c>
       <c r="H64" s="22" t="s">
-        <v>539</v>
+        <v>554</v>
       </c>
       <c r="I64" s="22" t="s">
-        <v>540</v>
+        <v>555</v>
       </c>
       <c r="J64" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K64" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L64" s="22" t="s">
-        <v>541</v>
+        <v>556</v>
       </c>
     </row>
     <row r="65" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B65" s="21" t="s">
-        <v>542</v>
+        <v>557</v>
       </c>
       <c r="C65" s="22" t="s">
         <v>59</v>
       </c>
       <c r="D65" s="22" t="s">
-        <v>543</v>
+        <v>558</v>
       </c>
       <c r="E65" s="22" t="s">
-        <v>544</v>
+        <v>559</v>
       </c>
       <c r="F65" s="22" t="s">
-        <v>545</v>
+        <v>560</v>
       </c>
       <c r="G65" s="22" t="s">
-        <v>546</v>
+        <v>561</v>
       </c>
       <c r="H65" s="22" t="s">
-        <v>547</v>
+        <v>562</v>
       </c>
       <c r="I65" s="22" t="s">
-        <v>548</v>
+        <v>563</v>
       </c>
       <c r="J65" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K65" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L65" s="22" t="s">
-        <v>549</v>
+        <v>564</v>
       </c>
     </row>
     <row r="66" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B66" s="21" t="s">
-        <v>550</v>
+        <v>565</v>
       </c>
       <c r="C66" s="22" t="s">
         <v>39</v>
       </c>
       <c r="D66" s="22" t="s">
-        <v>551</v>
+        <v>566</v>
       </c>
       <c r="E66" s="22" t="s">
-        <v>552</v>
+        <v>567</v>
       </c>
       <c r="F66" s="22" t="s">
-        <v>553</v>
+        <v>568</v>
       </c>
       <c r="G66" s="22" t="s">
-        <v>554</v>
+        <v>569</v>
       </c>
       <c r="H66" s="22" t="s">
-        <v>555</v>
+        <v>570</v>
       </c>
       <c r="I66" s="22" t="s">
-        <v>556</v>
+        <v>571</v>
       </c>
       <c r="J66" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K66" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L66" s="22" t="s">
-        <v>557</v>
+        <v>572</v>
       </c>
     </row>
     <row r="67" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B67" s="21" t="s">
-        <v>558</v>
+        <v>573</v>
       </c>
       <c r="C67" s="22" t="s">
         <v>37</v>
       </c>
       <c r="D67" s="22" t="s">
-        <v>559</v>
+        <v>574</v>
       </c>
       <c r="E67" s="22" t="s">
-        <v>560</v>
+        <v>575</v>
       </c>
       <c r="F67" s="22" t="s">
-        <v>561</v>
+        <v>576</v>
       </c>
       <c r="G67" s="22" t="s">
-        <v>562</v>
+        <v>577</v>
       </c>
       <c r="H67" s="22" t="s">
-        <v>563</v>
+        <v>578</v>
       </c>
       <c r="I67" s="22" t="s">
-        <v>564</v>
+        <v>579</v>
       </c>
       <c r="J67" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K67" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L67" s="22" t="s">
-        <v>565</v>
+        <v>580</v>
       </c>
     </row>
     <row r="68" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B68" s="21" t="s">
-        <v>566</v>
+        <v>581</v>
       </c>
       <c r="C68" s="22" t="s">
         <v>41</v>
       </c>
       <c r="D68" s="22" t="s">
-        <v>567</v>
+        <v>582</v>
       </c>
       <c r="E68" s="22" t="s">
-        <v>568</v>
+        <v>583</v>
       </c>
       <c r="F68" s="22" t="s">
-        <v>569</v>
+        <v>584</v>
       </c>
       <c r="G68" s="22" t="s">
-        <v>570</v>
+        <v>585</v>
       </c>
       <c r="H68" s="22" t="s">
-        <v>571</v>
+        <v>586</v>
       </c>
       <c r="I68" s="22" t="s">
-        <v>572</v>
+        <v>587</v>
       </c>
       <c r="J68" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K68" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L68" s="22" t="s">
-        <v>573</v>
+        <v>588</v>
       </c>
     </row>
     <row r="69" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B69" s="21" t="s">
-        <v>574</v>
+        <v>589</v>
       </c>
       <c r="C69" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D69" s="22" t="s">
-        <v>575</v>
+        <v>590</v>
       </c>
       <c r="E69" s="22" t="s">
-        <v>576</v>
+        <v>591</v>
       </c>
       <c r="F69" s="22" t="s">
-        <v>577</v>
+        <v>592</v>
       </c>
       <c r="G69" s="22" t="s">
-        <v>578</v>
+        <v>593</v>
       </c>
       <c r="H69" s="22" t="s">
-        <v>579</v>
+        <v>594</v>
       </c>
       <c r="I69" s="22" t="s">
-        <v>580</v>
+        <v>595</v>
       </c>
       <c r="J69" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K69" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L69" s="22" t="s">
-        <v>581</v>
+        <v>596</v>
       </c>
     </row>
     <row r="70" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B70" s="21" t="s">
-        <v>582</v>
+        <v>597</v>
       </c>
       <c r="C70" s="22" t="s">
         <v>34</v>
       </c>
       <c r="D70" s="22" t="s">
-        <v>583</v>
+        <v>598</v>
       </c>
       <c r="E70" s="22" t="s">
-        <v>584</v>
+        <v>599</v>
       </c>
       <c r="F70" s="22" t="s">
-        <v>585</v>
+        <v>600</v>
       </c>
       <c r="G70" s="22" t="s">
-        <v>586</v>
+        <v>601</v>
       </c>
       <c r="H70" s="22" t="s">
-        <v>587</v>
+        <v>602</v>
       </c>
       <c r="I70" s="22" t="s">
-        <v>588</v>
+        <v>603</v>
       </c>
       <c r="J70" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K70" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L70" s="22" t="s">
-        <v>589</v>
+        <v>604</v>
       </c>
     </row>
     <row r="71" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B71" s="21" t="s">
-        <v>590</v>
+        <v>605</v>
       </c>
       <c r="C71" s="22" t="s">
         <v>55</v>
       </c>
       <c r="D71" s="22" t="s">
-        <v>591</v>
+        <v>606</v>
       </c>
       <c r="E71" s="22" t="s">
-        <v>592</v>
+        <v>607</v>
       </c>
       <c r="F71" s="22" t="s">
-        <v>593</v>
+        <v>608</v>
       </c>
       <c r="G71" s="22" t="s">
-        <v>594</v>
+        <v>609</v>
       </c>
       <c r="H71" s="22" t="s">
-        <v>595</v>
+        <v>610</v>
       </c>
       <c r="I71" s="22" t="s">
-        <v>596</v>
+        <v>611</v>
       </c>
       <c r="J71" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K71" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L71" s="22" t="s">
-        <v>597</v>
+        <v>612</v>
       </c>
     </row>
     <row r="72" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B72" s="21" t="s">
-        <v>598</v>
+        <v>613</v>
       </c>
       <c r="C72" s="22" t="s">
         <v>32</v>
       </c>
       <c r="D72" s="22" t="s">
-        <v>599</v>
+        <v>614</v>
       </c>
       <c r="E72" s="22" t="s">
-        <v>600</v>
+        <v>615</v>
       </c>
       <c r="F72" s="22" t="s">
-        <v>601</v>
+        <v>616</v>
       </c>
       <c r="G72" s="22" t="s">
-        <v>602</v>
+        <v>617</v>
       </c>
       <c r="H72" s="22" t="s">
-        <v>603</v>
+        <v>618</v>
       </c>
       <c r="I72" s="22" t="s">
-        <v>604</v>
+        <v>619</v>
       </c>
       <c r="J72" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K72" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L72" s="22" t="s">
-        <v>605</v>
+        <v>620</v>
       </c>
     </row>
     <row r="73" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B73" s="21" t="s">
-        <v>606</v>
+        <v>621</v>
       </c>
       <c r="C73" s="22" t="s">
         <v>48</v>
       </c>
       <c r="D73" s="22" t="s">
-        <v>607</v>
+        <v>622</v>
       </c>
       <c r="E73" s="22" t="s">
-        <v>608</v>
+        <v>623</v>
       </c>
       <c r="F73" s="22" t="s">
-        <v>609</v>
+        <v>624</v>
       </c>
       <c r="G73" s="22" t="s">
-        <v>610</v>
+        <v>625</v>
       </c>
       <c r="H73" s="22" t="s">
-        <v>611</v>
+        <v>626</v>
       </c>
       <c r="I73" s="22" t="s">
-        <v>612</v>
+        <v>627</v>
       </c>
       <c r="J73" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K73" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L73" s="22" t="s">
-        <v>613</v>
+        <v>628</v>
       </c>
     </row>
     <row r="74" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B74" s="21" t="s">
-        <v>614</v>
+        <v>629</v>
       </c>
       <c r="C74" s="22" t="s">
         <v>26</v>
       </c>
       <c r="D74" s="22" t="s">
-        <v>615</v>
+        <v>630</v>
       </c>
       <c r="E74" s="22" t="s">
-        <v>616</v>
+        <v>631</v>
       </c>
       <c r="F74" s="22" t="s">
-        <v>617</v>
+        <v>632</v>
       </c>
       <c r="G74" s="22" t="s">
-        <v>618</v>
+        <v>633</v>
       </c>
       <c r="H74" s="22" t="s">
-        <v>619</v>
+        <v>634</v>
       </c>
       <c r="I74" s="22" t="s">
-        <v>620</v>
+        <v>635</v>
       </c>
       <c r="J74" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K74" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L74" s="22" t="s">
-        <v>621</v>
+        <v>636</v>
       </c>
     </row>
     <row r="75" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B75" s="21" t="s">
-        <v>622</v>
+        <v>637</v>
       </c>
       <c r="C75" s="22" t="s">
         <v>59</v>
       </c>
       <c r="D75" s="22" t="s">
-        <v>623</v>
+        <v>638</v>
       </c>
       <c r="E75" s="22" t="s">
-        <v>624</v>
+        <v>639</v>
       </c>
       <c r="F75" s="22" t="s">
-        <v>625</v>
+        <v>640</v>
       </c>
       <c r="G75" s="22" t="s">
-        <v>626</v>
+        <v>641</v>
       </c>
       <c r="H75" s="22" t="s">
-        <v>627</v>
+        <v>642</v>
       </c>
       <c r="I75" s="22" t="s">
-        <v>628</v>
+        <v>643</v>
       </c>
       <c r="J75" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K75" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L75" s="22" t="s">
-        <v>629</v>
+        <v>644</v>
       </c>
     </row>
     <row r="76" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B76" s="21" t="s">
-        <v>630</v>
+        <v>645</v>
       </c>
       <c r="C76" s="22" t="s">
         <v>59</v>
       </c>
       <c r="D76" s="22" t="s">
-        <v>631</v>
+        <v>646</v>
       </c>
       <c r="E76" s="22" t="s">
-        <v>632</v>
+        <v>647</v>
       </c>
       <c r="F76" s="22" t="s">
-        <v>633</v>
+        <v>648</v>
       </c>
       <c r="G76" s="22" t="s">
-        <v>634</v>
+        <v>649</v>
       </c>
       <c r="H76" s="22" t="s">
-        <v>635</v>
+        <v>650</v>
       </c>
       <c r="I76" s="22" t="s">
-        <v>636</v>
+        <v>651</v>
       </c>
       <c r="J76" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K76" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L76" s="22" t="s">
-        <v>637</v>
+        <v>652</v>
       </c>
     </row>
     <row r="77" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B77" s="21" t="s">
-        <v>638</v>
+        <v>653</v>
       </c>
       <c r="C77" s="22" t="s">
         <v>57</v>
       </c>
       <c r="D77" s="22" t="s">
-        <v>639</v>
+        <v>654</v>
       </c>
       <c r="E77" s="22" t="s">
-        <v>640</v>
+        <v>655</v>
       </c>
       <c r="F77" s="22" t="s">
-        <v>641</v>
+        <v>656</v>
       </c>
       <c r="G77" s="22" t="s">
-        <v>642</v>
+        <v>657</v>
       </c>
       <c r="H77" s="22" t="s">
-        <v>643</v>
+        <v>658</v>
       </c>
       <c r="I77" s="22" t="s">
-        <v>644</v>
+        <v>659</v>
       </c>
       <c r="J77" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K77" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L77" s="22" t="s">
-        <v>645</v>
+        <v>660</v>
       </c>
     </row>
     <row r="78" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B78" s="21" t="s">
-        <v>646</v>
+        <v>661</v>
       </c>
       <c r="C78" s="22" t="s">
         <v>57</v>
       </c>
       <c r="D78" s="22" t="s">
-        <v>647</v>
+        <v>662</v>
       </c>
       <c r="E78" s="22" t="s">
-        <v>640</v>
+        <v>655</v>
       </c>
       <c r="F78" s="22" t="s">
-        <v>648</v>
+        <v>663</v>
       </c>
       <c r="G78" s="22" t="s">
-        <v>649</v>
+        <v>664</v>
       </c>
       <c r="H78" s="22" t="s">
-        <v>650</v>
+        <v>665</v>
       </c>
       <c r="I78" s="22" t="s">
-        <v>651</v>
+        <v>666</v>
       </c>
       <c r="J78" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K78" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L78" s="22" t="s">
-        <v>652</v>
+        <v>667</v>
       </c>
     </row>
     <row r="79" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B79" s="21" t="s">
-        <v>653</v>
+        <v>668</v>
       </c>
       <c r="C79" s="22" t="s">
         <v>59</v>
       </c>
       <c r="D79" s="22" t="s">
-        <v>654</v>
+        <v>669</v>
       </c>
       <c r="E79" s="22" t="s">
-        <v>655</v>
+        <v>670</v>
       </c>
       <c r="F79" s="22" t="s">
-        <v>656</v>
+        <v>671</v>
       </c>
       <c r="G79" s="22" t="s">
-        <v>657</v>
+        <v>672</v>
       </c>
       <c r="H79" s="22" t="s">
-        <v>658</v>
+        <v>673</v>
       </c>
       <c r="I79" s="22" t="s">
-        <v>659</v>
+        <v>674</v>
       </c>
       <c r="J79" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K79" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L79" s="22" t="s">
-        <v>660</v>
+        <v>675</v>
       </c>
     </row>
     <row r="80" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B80" s="21" t="s">
-        <v>661</v>
+        <v>676</v>
       </c>
       <c r="C80" s="22" t="s">
         <v>59</v>
       </c>
       <c r="D80" s="22" t="s">
-        <v>662</v>
+        <v>677</v>
       </c>
       <c r="E80" s="22" t="s">
-        <v>663</v>
+        <v>678</v>
       </c>
       <c r="F80" s="22" t="s">
-        <v>664</v>
+        <v>679</v>
       </c>
       <c r="G80" s="22" t="s">
-        <v>665</v>
+        <v>680</v>
       </c>
       <c r="H80" s="22" t="s">
-        <v>666</v>
+        <v>681</v>
       </c>
       <c r="I80" s="22" t="s">
-        <v>667</v>
+        <v>682</v>
       </c>
       <c r="J80" s="23" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="K80" s="24" t="s">
         <v>20</v>
       </c>
       <c r="L80" s="22" t="s">
-        <v>668</v>
+        <v>683</v>
+      </c>
+    </row>
+    <row r="81" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B81" s="21" t="s">
+        <v>684</v>
+      </c>
+      <c r="C81" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="D81" s="22" t="s">
+        <v>685</v>
+      </c>
+      <c r="E81" s="22" t="s">
+        <v>686</v>
+      </c>
+      <c r="F81" s="22" t="s">
+        <v>687</v>
+      </c>
+      <c r="G81" s="22" t="s">
+        <v>688</v>
+      </c>
+      <c r="H81" s="22" t="s">
+        <v>689</v>
+      </c>
+      <c r="I81" s="22" t="s">
+        <v>690</v>
+      </c>
+      <c r="J81" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="K81" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L81" s="22" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="82" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B82" s="21" t="s">
+        <v>692</v>
+      </c>
+      <c r="C82" s="22" t="s">
+        <v>64</v>
+      </c>
+      <c r="D82" s="22" t="s">
+        <v>693</v>
+      </c>
+      <c r="E82" s="22" t="s">
+        <v>694</v>
+      </c>
+      <c r="F82" s="22" t="s">
+        <v>695</v>
+      </c>
+      <c r="G82" s="22" t="s">
+        <v>696</v>
+      </c>
+      <c r="H82" s="22" t="s">
+        <v>697</v>
+      </c>
+      <c r="I82" s="22" t="s">
+        <v>698</v>
+      </c>
+      <c r="J82" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="K82" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L82" s="22" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="83" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B83" s="21" t="s">
+        <v>700</v>
+      </c>
+      <c r="C83" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="D83" s="22" t="s">
+        <v>701</v>
+      </c>
+      <c r="E83" s="22" t="s">
+        <v>702</v>
+      </c>
+      <c r="F83" s="22" t="s">
+        <v>703</v>
+      </c>
+      <c r="G83" s="22" t="s">
+        <v>704</v>
+      </c>
+      <c r="H83" s="22" t="s">
+        <v>705</v>
+      </c>
+      <c r="I83" s="22" t="s">
+        <v>706</v>
+      </c>
+      <c r="J83" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="K83" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L83" s="22" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="84" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B84" s="21" t="s">
+        <v>708</v>
+      </c>
+      <c r="C84" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="D84" s="22" t="s">
+        <v>709</v>
+      </c>
+      <c r="E84" s="22" t="s">
+        <v>710</v>
+      </c>
+      <c r="F84" s="22" t="s">
+        <v>711</v>
+      </c>
+      <c r="G84" s="22" t="s">
+        <v>712</v>
+      </c>
+      <c r="H84" s="22" t="s">
+        <v>713</v>
+      </c>
+      <c r="I84" s="22" t="s">
+        <v>714</v>
+      </c>
+      <c r="J84" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="K84" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L84" s="22" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="85" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B85" s="21" t="s">
+        <v>716</v>
+      </c>
+      <c r="C85" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="D85" s="22" t="s">
+        <v>717</v>
+      </c>
+      <c r="E85" s="22" t="s">
+        <v>303</v>
+      </c>
+      <c r="F85" s="22" t="s">
+        <v>718</v>
+      </c>
+      <c r="G85" s="22" t="s">
+        <v>719</v>
+      </c>
+      <c r="H85" s="22" t="s">
+        <v>720</v>
+      </c>
+      <c r="I85" s="22" t="s">
+        <v>721</v>
+      </c>
+      <c r="J85" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="K85" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L85" s="22" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="86" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B86" s="21" t="s">
+        <v>723</v>
+      </c>
+      <c r="C86" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="D86" s="22" t="s">
+        <v>724</v>
+      </c>
+      <c r="E86" s="22" t="s">
+        <v>725</v>
+      </c>
+      <c r="F86" s="22" t="s">
+        <v>726</v>
+      </c>
+      <c r="G86" s="22" t="s">
+        <v>727</v>
+      </c>
+      <c r="H86" s="22" t="s">
+        <v>728</v>
+      </c>
+      <c r="I86" s="22" t="s">
+        <v>729</v>
+      </c>
+      <c r="J86" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="K86" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L86" s="22" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="87" ht="42" customHeight="1" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B87" s="21" t="s">
+        <v>731</v>
+      </c>
+      <c r="C87" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="D87" s="22" t="s">
+        <v>732</v>
+      </c>
+      <c r="E87" s="22" t="s">
+        <v>733</v>
+      </c>
+      <c r="F87" s="22" t="s">
+        <v>734</v>
+      </c>
+      <c r="G87" s="22" t="s">
+        <v>735</v>
+      </c>
+      <c r="H87" s="22" t="s">
+        <v>736</v>
+      </c>
+      <c r="I87" s="22" t="s">
+        <v>737</v>
+      </c>
+      <c r="J87" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="K87" s="24" t="s">
+        <v>20</v>
+      </c>
+      <c r="L87" s="22" t="s">
+        <v>738</v>
       </c>
     </row>
   </sheetData>

</xml_diff>